<commit_message>
W05 SAT: the discussion guide, the provenance, and the leak and level fixes
The guide runs the 300-minute Saturday with the ME1 window held without marks,
day or slot, answers the row's nine anchors as reasoning with two follow-ups
each, and previews Build 2's five seeds. The paper no longer names the duration
trap before Q12, each bank blank prints last in its part, Q15 and Q23 join a
cause or rule to its consequence, and the levels read 4, 9 and 13 by the
exercise-builder bar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TK2R2uaDnJSEF8EjfT4zg9
</commit_message>
<xml_diff>
--- a/content/W05/SAT/answer-key/C2_W05_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W05/SAT/answer-key/C2_W05_SAT_item_analysis_TRAINER.xlsx
@@ -617,107 +617,107 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>[D]</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>[F]</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>[S]</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>[F]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>[D]</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>[F]</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>[F]</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>[S]</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>[S]</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>[F]</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>[F]</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>[D]</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>[S]</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>[S]</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>[S]</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>[D]</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>[S]</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>[S]</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>[S]</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>[F]</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>[F]</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>[S]</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>[F]</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>[S]</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>[F]</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>[F]</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>[D]</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -2675,12 +2675,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fill in the blank</t>
+          <t>One correct option</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G5">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>One correct option</t>
+          <t>True or false</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2745,12 +2745,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>[S]</t>
+          <t>[D]</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G6">
@@ -2795,22 +2795,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>True or false</t>
+          <t>One correct option</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[D]</t>
+          <t>[F]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>d</t>
         </is>
       </c>
       <c r="G7">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>One correct option</t>
+          <t>More than one correct</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2865,12 +2865,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[S]</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>a, d</t>
         </is>
       </c>
       <c r="G8">
@@ -2915,12 +2915,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>More than one correct</t>
+          <t>Fill in the blank</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>a, d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G9">
@@ -2975,22 +2975,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fill in the blank</t>
+          <t>True or false</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>[S]</t>
+          <t>[F]</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>d</t>
         </is>
       </c>
       <c r="G10">
@@ -3035,22 +3035,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>True or false</t>
+          <t>Applied maths</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[S]</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>Precision 174 / 268 = 0.65; recall 174 / 928 = 0.19; F1 = 2 x 174 / (2 x 174 + 94 + 754) = 348 / 1,196 = 0.29.</t>
         </is>
       </c>
       <c r="G11">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Precision 174 / 268 = 0.65; recall 174 / 928 = 0.19; F1 = 2 x 174 / (2 x 174 + 94 + 754) = 348 / 1,196 = 0.29.</t>
+          <t>Call when p x 1,200 &gt; (1 - p) x 40, so p &gt; 40 / 1,240 = 1 / 31, about 0.032; the line moves down from 0.5 and recall leads.</t>
         </is>
       </c>
       <c r="G12">
@@ -3155,12 +3155,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Applied maths</t>
+          <t>One correct option</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Call when p x 1,200 &gt; (1 - p) x 40, so p &gt; 40 / 1,240 = 1 / 31, about 0.032; the line moves down from 0.5 and recall leads.</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G13">
@@ -3225,12 +3225,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>[S]</t>
+          <t>[D]</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G14">
@@ -3275,22 +3275,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>One correct option</t>
+          <t>Fill in the blank</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>[D]</t>
+          <t>[S]</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G15">
@@ -3335,12 +3335,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fill in the blank</t>
+          <t>One correct option</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>One correct option</t>
+          <t>More than one correct</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b, c, d</t>
         </is>
       </c>
       <c r="G17">
@@ -3455,22 +3455,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>More than one correct</t>
+          <t>True or false</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>[S]</t>
+          <t>[F]</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>b, c, d</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G18">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>True or false</t>
+          <t>One correct option</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>d</t>
         </is>
       </c>
       <c r="G19">
@@ -3575,22 +3575,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>One correct option</t>
+          <t>Fill in the blank</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[S]</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G20">
@@ -3635,12 +3635,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Fill in the blank</t>
+          <t>One correct option</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Fill in the blank</t>
+          <t>More than one correct</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>a, b, d</t>
         </is>
       </c>
       <c r="G22">
@@ -3765,12 +3765,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>[S]</t>
+          <t>[F]</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G23">
@@ -3815,22 +3815,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>More than one correct</t>
+          <t>True or false</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[D]</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>a, b, d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G24">
@@ -3875,22 +3875,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>One correct option</t>
+          <t>Fill in the blank</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[S]</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G25">
@@ -3935,22 +3935,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>True or false</t>
+          <t>Fill in the blank</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>[D]</t>
+          <t>[F]</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>d</t>
         </is>
       </c>
       <c r="G26">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">

</xml_diff>

<commit_message>
W05 SAT: the blind sitting's fix pass
Two statements now read True, the memo boxes, Q10's precision and the top
1,000 row no longer answer other items, banks 4 and 5 fold into the items
that test them, Q13 and Q24 each take two steps, five options read one way
only, and the levels are relabelled by the exercise-builder bar: 24 items at
57 minutes, 3 easy, 14 medium and 7 hard. The sources file records each
finding and its change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TK2R2uaDnJSEF8EjfT4zg9
</commit_message>
<xml_diff>
--- a/content/W05/SAT/answer-key/C2_W05_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W05/SAT/answer-key/C2_W05_SAT_item_analysis_TRAINER.xlsx
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD43"/>
+  <dimension ref="A1:AB43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -586,10 +586,10 @@
         <v>4</v>
       </c>
       <c r="V2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X2" t="n">
         <v>5</v>
@@ -597,12 +597,6 @@
       <c r="Y2" t="n">
         <v>5</v>
       </c>
-      <c r="Z2" t="n">
-        <v>5</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -712,30 +706,20 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>[S]</t>
+          <t>[F]</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[D]</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[D]</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
-        <is>
-          <t>[D]</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>[D]</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
         <is>
           <t>[D]</t>
         </is>
@@ -869,25 +853,15 @@
       </c>
       <c r="Z4" s="4" t="inlineStr">
         <is>
-          <t>Q25</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="AA4" s="4" t="inlineStr">
         <is>
-          <t>Q26</t>
+          <t>Answered</t>
         </is>
       </c>
       <c r="AB4" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="AC4" s="4" t="inlineStr">
-        <is>
-          <t>Answered</t>
-        </is>
-      </c>
-      <c r="AD4" s="4" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
@@ -921,18 +895,16 @@
       <c r="W5" s="5" t="n"/>
       <c r="X5" s="5" t="n"/>
       <c r="Y5" s="5" t="n"/>
-      <c r="Z5" s="5" t="n"/>
-      <c r="AA5" s="5" t="n"/>
+      <c r="Z5">
+        <f>IF(COUNT(B5:Y5)=0,"",SUM(B5:Y5))</f>
+        <v/>
+      </c>
+      <c r="AA5">
+        <f>COUNT(B5:Y5)</f>
+        <v/>
+      </c>
       <c r="AB5">
-        <f>IF(COUNT(B5:AA5)=0,"",SUM(B5:AA5))</f>
-        <v/>
-      </c>
-      <c r="AC5">
-        <f>COUNT(B5:AA5)</f>
-        <v/>
-      </c>
-      <c r="AD5">
-        <f>IF(OR(AB5="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB5,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB5,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z5="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z5,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z5,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -964,18 +936,16 @@
       <c r="W6" s="5" t="n"/>
       <c r="X6" s="5" t="n"/>
       <c r="Y6" s="5" t="n"/>
-      <c r="Z6" s="5" t="n"/>
-      <c r="AA6" s="5" t="n"/>
+      <c r="Z6">
+        <f>IF(COUNT(B6:Y6)=0,"",SUM(B6:Y6))</f>
+        <v/>
+      </c>
+      <c r="AA6">
+        <f>COUNT(B6:Y6)</f>
+        <v/>
+      </c>
       <c r="AB6">
-        <f>IF(COUNT(B6:AA6)=0,"",SUM(B6:AA6))</f>
-        <v/>
-      </c>
-      <c r="AC6">
-        <f>COUNT(B6:AA6)</f>
-        <v/>
-      </c>
-      <c r="AD6">
-        <f>IF(OR(AB6="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB6,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB6,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z6="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z6,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z6,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1007,18 +977,16 @@
       <c r="W7" s="5" t="n"/>
       <c r="X7" s="5" t="n"/>
       <c r="Y7" s="5" t="n"/>
-      <c r="Z7" s="5" t="n"/>
-      <c r="AA7" s="5" t="n"/>
+      <c r="Z7">
+        <f>IF(COUNT(B7:Y7)=0,"",SUM(B7:Y7))</f>
+        <v/>
+      </c>
+      <c r="AA7">
+        <f>COUNT(B7:Y7)</f>
+        <v/>
+      </c>
       <c r="AB7">
-        <f>IF(COUNT(B7:AA7)=0,"",SUM(B7:AA7))</f>
-        <v/>
-      </c>
-      <c r="AC7">
-        <f>COUNT(B7:AA7)</f>
-        <v/>
-      </c>
-      <c r="AD7">
-        <f>IF(OR(AB7="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB7,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB7,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z7="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z7,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z7,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1050,18 +1018,16 @@
       <c r="W8" s="5" t="n"/>
       <c r="X8" s="5" t="n"/>
       <c r="Y8" s="5" t="n"/>
-      <c r="Z8" s="5" t="n"/>
-      <c r="AA8" s="5" t="n"/>
+      <c r="Z8">
+        <f>IF(COUNT(B8:Y8)=0,"",SUM(B8:Y8))</f>
+        <v/>
+      </c>
+      <c r="AA8">
+        <f>COUNT(B8:Y8)</f>
+        <v/>
+      </c>
       <c r="AB8">
-        <f>IF(COUNT(B8:AA8)=0,"",SUM(B8:AA8))</f>
-        <v/>
-      </c>
-      <c r="AC8">
-        <f>COUNT(B8:AA8)</f>
-        <v/>
-      </c>
-      <c r="AD8">
-        <f>IF(OR(AB8="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB8,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB8,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z8="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z8,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z8,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1093,18 +1059,16 @@
       <c r="W9" s="5" t="n"/>
       <c r="X9" s="5" t="n"/>
       <c r="Y9" s="5" t="n"/>
-      <c r="Z9" s="5" t="n"/>
-      <c r="AA9" s="5" t="n"/>
+      <c r="Z9">
+        <f>IF(COUNT(B9:Y9)=0,"",SUM(B9:Y9))</f>
+        <v/>
+      </c>
+      <c r="AA9">
+        <f>COUNT(B9:Y9)</f>
+        <v/>
+      </c>
       <c r="AB9">
-        <f>IF(COUNT(B9:AA9)=0,"",SUM(B9:AA9))</f>
-        <v/>
-      </c>
-      <c r="AC9">
-        <f>COUNT(B9:AA9)</f>
-        <v/>
-      </c>
-      <c r="AD9">
-        <f>IF(OR(AB9="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB9,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB9,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z9="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z9,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z9,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1136,18 +1100,16 @@
       <c r="W10" s="5" t="n"/>
       <c r="X10" s="5" t="n"/>
       <c r="Y10" s="5" t="n"/>
-      <c r="Z10" s="5" t="n"/>
-      <c r="AA10" s="5" t="n"/>
+      <c r="Z10">
+        <f>IF(COUNT(B10:Y10)=0,"",SUM(B10:Y10))</f>
+        <v/>
+      </c>
+      <c r="AA10">
+        <f>COUNT(B10:Y10)</f>
+        <v/>
+      </c>
       <c r="AB10">
-        <f>IF(COUNT(B10:AA10)=0,"",SUM(B10:AA10))</f>
-        <v/>
-      </c>
-      <c r="AC10">
-        <f>COUNT(B10:AA10)</f>
-        <v/>
-      </c>
-      <c r="AD10">
-        <f>IF(OR(AB10="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB10,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB10,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z10="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z10,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z10,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1179,18 +1141,16 @@
       <c r="W11" s="5" t="n"/>
       <c r="X11" s="5" t="n"/>
       <c r="Y11" s="5" t="n"/>
-      <c r="Z11" s="5" t="n"/>
-      <c r="AA11" s="5" t="n"/>
+      <c r="Z11">
+        <f>IF(COUNT(B11:Y11)=0,"",SUM(B11:Y11))</f>
+        <v/>
+      </c>
+      <c r="AA11">
+        <f>COUNT(B11:Y11)</f>
+        <v/>
+      </c>
       <c r="AB11">
-        <f>IF(COUNT(B11:AA11)=0,"",SUM(B11:AA11))</f>
-        <v/>
-      </c>
-      <c r="AC11">
-        <f>COUNT(B11:AA11)</f>
-        <v/>
-      </c>
-      <c r="AD11">
-        <f>IF(OR(AB11="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB11,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB11,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z11="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z11,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z11,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1222,18 +1182,16 @@
       <c r="W12" s="5" t="n"/>
       <c r="X12" s="5" t="n"/>
       <c r="Y12" s="5" t="n"/>
-      <c r="Z12" s="5" t="n"/>
-      <c r="AA12" s="5" t="n"/>
+      <c r="Z12">
+        <f>IF(COUNT(B12:Y12)=0,"",SUM(B12:Y12))</f>
+        <v/>
+      </c>
+      <c r="AA12">
+        <f>COUNT(B12:Y12)</f>
+        <v/>
+      </c>
       <c r="AB12">
-        <f>IF(COUNT(B12:AA12)=0,"",SUM(B12:AA12))</f>
-        <v/>
-      </c>
-      <c r="AC12">
-        <f>COUNT(B12:AA12)</f>
-        <v/>
-      </c>
-      <c r="AD12">
-        <f>IF(OR(AB12="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB12,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB12,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z12="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z12,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z12,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1265,18 +1223,16 @@
       <c r="W13" s="5" t="n"/>
       <c r="X13" s="5" t="n"/>
       <c r="Y13" s="5" t="n"/>
-      <c r="Z13" s="5" t="n"/>
-      <c r="AA13" s="5" t="n"/>
+      <c r="Z13">
+        <f>IF(COUNT(B13:Y13)=0,"",SUM(B13:Y13))</f>
+        <v/>
+      </c>
+      <c r="AA13">
+        <f>COUNT(B13:Y13)</f>
+        <v/>
+      </c>
       <c r="AB13">
-        <f>IF(COUNT(B13:AA13)=0,"",SUM(B13:AA13))</f>
-        <v/>
-      </c>
-      <c r="AC13">
-        <f>COUNT(B13:AA13)</f>
-        <v/>
-      </c>
-      <c r="AD13">
-        <f>IF(OR(AB13="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB13,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB13,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z13="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z13,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z13,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1308,18 +1264,16 @@
       <c r="W14" s="5" t="n"/>
       <c r="X14" s="5" t="n"/>
       <c r="Y14" s="5" t="n"/>
-      <c r="Z14" s="5" t="n"/>
-      <c r="AA14" s="5" t="n"/>
+      <c r="Z14">
+        <f>IF(COUNT(B14:Y14)=0,"",SUM(B14:Y14))</f>
+        <v/>
+      </c>
+      <c r="AA14">
+        <f>COUNT(B14:Y14)</f>
+        <v/>
+      </c>
       <c r="AB14">
-        <f>IF(COUNT(B14:AA14)=0,"",SUM(B14:AA14))</f>
-        <v/>
-      </c>
-      <c r="AC14">
-        <f>COUNT(B14:AA14)</f>
-        <v/>
-      </c>
-      <c r="AD14">
-        <f>IF(OR(AB14="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB14,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB14,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z14="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z14,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z14,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1351,18 +1305,16 @@
       <c r="W15" s="5" t="n"/>
       <c r="X15" s="5" t="n"/>
       <c r="Y15" s="5" t="n"/>
-      <c r="Z15" s="5" t="n"/>
-      <c r="AA15" s="5" t="n"/>
+      <c r="Z15">
+        <f>IF(COUNT(B15:Y15)=0,"",SUM(B15:Y15))</f>
+        <v/>
+      </c>
+      <c r="AA15">
+        <f>COUNT(B15:Y15)</f>
+        <v/>
+      </c>
       <c r="AB15">
-        <f>IF(COUNT(B15:AA15)=0,"",SUM(B15:AA15))</f>
-        <v/>
-      </c>
-      <c r="AC15">
-        <f>COUNT(B15:AA15)</f>
-        <v/>
-      </c>
-      <c r="AD15">
-        <f>IF(OR(AB15="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB15,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB15,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z15="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z15,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z15,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1394,18 +1346,16 @@
       <c r="W16" s="5" t="n"/>
       <c r="X16" s="5" t="n"/>
       <c r="Y16" s="5" t="n"/>
-      <c r="Z16" s="5" t="n"/>
-      <c r="AA16" s="5" t="n"/>
+      <c r="Z16">
+        <f>IF(COUNT(B16:Y16)=0,"",SUM(B16:Y16))</f>
+        <v/>
+      </c>
+      <c r="AA16">
+        <f>COUNT(B16:Y16)</f>
+        <v/>
+      </c>
       <c r="AB16">
-        <f>IF(COUNT(B16:AA16)=0,"",SUM(B16:AA16))</f>
-        <v/>
-      </c>
-      <c r="AC16">
-        <f>COUNT(B16:AA16)</f>
-        <v/>
-      </c>
-      <c r="AD16">
-        <f>IF(OR(AB16="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB16,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB16,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z16="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z16,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z16,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1437,18 +1387,16 @@
       <c r="W17" s="5" t="n"/>
       <c r="X17" s="5" t="n"/>
       <c r="Y17" s="5" t="n"/>
-      <c r="Z17" s="5" t="n"/>
-      <c r="AA17" s="5" t="n"/>
+      <c r="Z17">
+        <f>IF(COUNT(B17:Y17)=0,"",SUM(B17:Y17))</f>
+        <v/>
+      </c>
+      <c r="AA17">
+        <f>COUNT(B17:Y17)</f>
+        <v/>
+      </c>
       <c r="AB17">
-        <f>IF(COUNT(B17:AA17)=0,"",SUM(B17:AA17))</f>
-        <v/>
-      </c>
-      <c r="AC17">
-        <f>COUNT(B17:AA17)</f>
-        <v/>
-      </c>
-      <c r="AD17">
-        <f>IF(OR(AB17="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB17,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB17,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z17="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z17,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z17,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1480,18 +1428,16 @@
       <c r="W18" s="5" t="n"/>
       <c r="X18" s="5" t="n"/>
       <c r="Y18" s="5" t="n"/>
-      <c r="Z18" s="5" t="n"/>
-      <c r="AA18" s="5" t="n"/>
+      <c r="Z18">
+        <f>IF(COUNT(B18:Y18)=0,"",SUM(B18:Y18))</f>
+        <v/>
+      </c>
+      <c r="AA18">
+        <f>COUNT(B18:Y18)</f>
+        <v/>
+      </c>
       <c r="AB18">
-        <f>IF(COUNT(B18:AA18)=0,"",SUM(B18:AA18))</f>
-        <v/>
-      </c>
-      <c r="AC18">
-        <f>COUNT(B18:AA18)</f>
-        <v/>
-      </c>
-      <c r="AD18">
-        <f>IF(OR(AB18="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB18,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB18,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z18="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z18,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z18,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1523,18 +1469,16 @@
       <c r="W19" s="5" t="n"/>
       <c r="X19" s="5" t="n"/>
       <c r="Y19" s="5" t="n"/>
-      <c r="Z19" s="5" t="n"/>
-      <c r="AA19" s="5" t="n"/>
+      <c r="Z19">
+        <f>IF(COUNT(B19:Y19)=0,"",SUM(B19:Y19))</f>
+        <v/>
+      </c>
+      <c r="AA19">
+        <f>COUNT(B19:Y19)</f>
+        <v/>
+      </c>
       <c r="AB19">
-        <f>IF(COUNT(B19:AA19)=0,"",SUM(B19:AA19))</f>
-        <v/>
-      </c>
-      <c r="AC19">
-        <f>COUNT(B19:AA19)</f>
-        <v/>
-      </c>
-      <c r="AD19">
-        <f>IF(OR(AB19="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB19,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB19,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z19="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z19,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z19,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1566,18 +1510,16 @@
       <c r="W20" s="5" t="n"/>
       <c r="X20" s="5" t="n"/>
       <c r="Y20" s="5" t="n"/>
-      <c r="Z20" s="5" t="n"/>
-      <c r="AA20" s="5" t="n"/>
+      <c r="Z20">
+        <f>IF(COUNT(B20:Y20)=0,"",SUM(B20:Y20))</f>
+        <v/>
+      </c>
+      <c r="AA20">
+        <f>COUNT(B20:Y20)</f>
+        <v/>
+      </c>
       <c r="AB20">
-        <f>IF(COUNT(B20:AA20)=0,"",SUM(B20:AA20))</f>
-        <v/>
-      </c>
-      <c r="AC20">
-        <f>COUNT(B20:AA20)</f>
-        <v/>
-      </c>
-      <c r="AD20">
-        <f>IF(OR(AB20="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB20,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB20,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z20="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z20,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z20,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1609,18 +1551,16 @@
       <c r="W21" s="5" t="n"/>
       <c r="X21" s="5" t="n"/>
       <c r="Y21" s="5" t="n"/>
-      <c r="Z21" s="5" t="n"/>
-      <c r="AA21" s="5" t="n"/>
+      <c r="Z21">
+        <f>IF(COUNT(B21:Y21)=0,"",SUM(B21:Y21))</f>
+        <v/>
+      </c>
+      <c r="AA21">
+        <f>COUNT(B21:Y21)</f>
+        <v/>
+      </c>
       <c r="AB21">
-        <f>IF(COUNT(B21:AA21)=0,"",SUM(B21:AA21))</f>
-        <v/>
-      </c>
-      <c r="AC21">
-        <f>COUNT(B21:AA21)</f>
-        <v/>
-      </c>
-      <c r="AD21">
-        <f>IF(OR(AB21="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB21,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB21,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z21="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z21,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z21,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1652,18 +1592,16 @@
       <c r="W22" s="5" t="n"/>
       <c r="X22" s="5" t="n"/>
       <c r="Y22" s="5" t="n"/>
-      <c r="Z22" s="5" t="n"/>
-      <c r="AA22" s="5" t="n"/>
+      <c r="Z22">
+        <f>IF(COUNT(B22:Y22)=0,"",SUM(B22:Y22))</f>
+        <v/>
+      </c>
+      <c r="AA22">
+        <f>COUNT(B22:Y22)</f>
+        <v/>
+      </c>
       <c r="AB22">
-        <f>IF(COUNT(B22:AA22)=0,"",SUM(B22:AA22))</f>
-        <v/>
-      </c>
-      <c r="AC22">
-        <f>COUNT(B22:AA22)</f>
-        <v/>
-      </c>
-      <c r="AD22">
-        <f>IF(OR(AB22="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB22,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB22,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z22="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z22,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z22,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1695,18 +1633,16 @@
       <c r="W23" s="5" t="n"/>
       <c r="X23" s="5" t="n"/>
       <c r="Y23" s="5" t="n"/>
-      <c r="Z23" s="5" t="n"/>
-      <c r="AA23" s="5" t="n"/>
+      <c r="Z23">
+        <f>IF(COUNT(B23:Y23)=0,"",SUM(B23:Y23))</f>
+        <v/>
+      </c>
+      <c r="AA23">
+        <f>COUNT(B23:Y23)</f>
+        <v/>
+      </c>
       <c r="AB23">
-        <f>IF(COUNT(B23:AA23)=0,"",SUM(B23:AA23))</f>
-        <v/>
-      </c>
-      <c r="AC23">
-        <f>COUNT(B23:AA23)</f>
-        <v/>
-      </c>
-      <c r="AD23">
-        <f>IF(OR(AB23="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB23,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB23,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z23="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z23,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z23,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1738,18 +1674,16 @@
       <c r="W24" s="5" t="n"/>
       <c r="X24" s="5" t="n"/>
       <c r="Y24" s="5" t="n"/>
-      <c r="Z24" s="5" t="n"/>
-      <c r="AA24" s="5" t="n"/>
+      <c r="Z24">
+        <f>IF(COUNT(B24:Y24)=0,"",SUM(B24:Y24))</f>
+        <v/>
+      </c>
+      <c r="AA24">
+        <f>COUNT(B24:Y24)</f>
+        <v/>
+      </c>
       <c r="AB24">
-        <f>IF(COUNT(B24:AA24)=0,"",SUM(B24:AA24))</f>
-        <v/>
-      </c>
-      <c r="AC24">
-        <f>COUNT(B24:AA24)</f>
-        <v/>
-      </c>
-      <c r="AD24">
-        <f>IF(OR(AB24="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB24,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB24,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z24="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z24,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z24,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1781,18 +1715,16 @@
       <c r="W25" s="5" t="n"/>
       <c r="X25" s="5" t="n"/>
       <c r="Y25" s="5" t="n"/>
-      <c r="Z25" s="5" t="n"/>
-      <c r="AA25" s="5" t="n"/>
+      <c r="Z25">
+        <f>IF(COUNT(B25:Y25)=0,"",SUM(B25:Y25))</f>
+        <v/>
+      </c>
+      <c r="AA25">
+        <f>COUNT(B25:Y25)</f>
+        <v/>
+      </c>
       <c r="AB25">
-        <f>IF(COUNT(B25:AA25)=0,"",SUM(B25:AA25))</f>
-        <v/>
-      </c>
-      <c r="AC25">
-        <f>COUNT(B25:AA25)</f>
-        <v/>
-      </c>
-      <c r="AD25">
-        <f>IF(OR(AB25="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB25,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB25,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z25="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z25,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z25,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1824,18 +1756,16 @@
       <c r="W26" s="5" t="n"/>
       <c r="X26" s="5" t="n"/>
       <c r="Y26" s="5" t="n"/>
-      <c r="Z26" s="5" t="n"/>
-      <c r="AA26" s="5" t="n"/>
+      <c r="Z26">
+        <f>IF(COUNT(B26:Y26)=0,"",SUM(B26:Y26))</f>
+        <v/>
+      </c>
+      <c r="AA26">
+        <f>COUNT(B26:Y26)</f>
+        <v/>
+      </c>
       <c r="AB26">
-        <f>IF(COUNT(B26:AA26)=0,"",SUM(B26:AA26))</f>
-        <v/>
-      </c>
-      <c r="AC26">
-        <f>COUNT(B26:AA26)</f>
-        <v/>
-      </c>
-      <c r="AD26">
-        <f>IF(OR(AB26="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB26,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB26,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z26="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z26,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z26,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1867,18 +1797,16 @@
       <c r="W27" s="5" t="n"/>
       <c r="X27" s="5" t="n"/>
       <c r="Y27" s="5" t="n"/>
-      <c r="Z27" s="5" t="n"/>
-      <c r="AA27" s="5" t="n"/>
+      <c r="Z27">
+        <f>IF(COUNT(B27:Y27)=0,"",SUM(B27:Y27))</f>
+        <v/>
+      </c>
+      <c r="AA27">
+        <f>COUNT(B27:Y27)</f>
+        <v/>
+      </c>
       <c r="AB27">
-        <f>IF(COUNT(B27:AA27)=0,"",SUM(B27:AA27))</f>
-        <v/>
-      </c>
-      <c r="AC27">
-        <f>COUNT(B27:AA27)</f>
-        <v/>
-      </c>
-      <c r="AD27">
-        <f>IF(OR(AB27="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB27,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB27,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z27="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z27,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z27,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1910,18 +1838,16 @@
       <c r="W28" s="5" t="n"/>
       <c r="X28" s="5" t="n"/>
       <c r="Y28" s="5" t="n"/>
-      <c r="Z28" s="5" t="n"/>
-      <c r="AA28" s="5" t="n"/>
+      <c r="Z28">
+        <f>IF(COUNT(B28:Y28)=0,"",SUM(B28:Y28))</f>
+        <v/>
+      </c>
+      <c r="AA28">
+        <f>COUNT(B28:Y28)</f>
+        <v/>
+      </c>
       <c r="AB28">
-        <f>IF(COUNT(B28:AA28)=0,"",SUM(B28:AA28))</f>
-        <v/>
-      </c>
-      <c r="AC28">
-        <f>COUNT(B28:AA28)</f>
-        <v/>
-      </c>
-      <c r="AD28">
-        <f>IF(OR(AB28="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB28,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB28,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z28="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z28,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z28,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1953,18 +1879,16 @@
       <c r="W29" s="5" t="n"/>
       <c r="X29" s="5" t="n"/>
       <c r="Y29" s="5" t="n"/>
-      <c r="Z29" s="5" t="n"/>
-      <c r="AA29" s="5" t="n"/>
+      <c r="Z29">
+        <f>IF(COUNT(B29:Y29)=0,"",SUM(B29:Y29))</f>
+        <v/>
+      </c>
+      <c r="AA29">
+        <f>COUNT(B29:Y29)</f>
+        <v/>
+      </c>
       <c r="AB29">
-        <f>IF(COUNT(B29:AA29)=0,"",SUM(B29:AA29))</f>
-        <v/>
-      </c>
-      <c r="AC29">
-        <f>COUNT(B29:AA29)</f>
-        <v/>
-      </c>
-      <c r="AD29">
-        <f>IF(OR(AB29="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB29,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB29,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z29="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z29,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z29,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1996,18 +1920,16 @@
       <c r="W30" s="5" t="n"/>
       <c r="X30" s="5" t="n"/>
       <c r="Y30" s="5" t="n"/>
-      <c r="Z30" s="5" t="n"/>
-      <c r="AA30" s="5" t="n"/>
+      <c r="Z30">
+        <f>IF(COUNT(B30:Y30)=0,"",SUM(B30:Y30))</f>
+        <v/>
+      </c>
+      <c r="AA30">
+        <f>COUNT(B30:Y30)</f>
+        <v/>
+      </c>
       <c r="AB30">
-        <f>IF(COUNT(B30:AA30)=0,"",SUM(B30:AA30))</f>
-        <v/>
-      </c>
-      <c r="AC30">
-        <f>COUNT(B30:AA30)</f>
-        <v/>
-      </c>
-      <c r="AD30">
-        <f>IF(OR(AB30="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB30,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB30,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z30="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z30,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z30,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2039,18 +1961,16 @@
       <c r="W31" s="5" t="n"/>
       <c r="X31" s="5" t="n"/>
       <c r="Y31" s="5" t="n"/>
-      <c r="Z31" s="5" t="n"/>
-      <c r="AA31" s="5" t="n"/>
+      <c r="Z31">
+        <f>IF(COUNT(B31:Y31)=0,"",SUM(B31:Y31))</f>
+        <v/>
+      </c>
+      <c r="AA31">
+        <f>COUNT(B31:Y31)</f>
+        <v/>
+      </c>
       <c r="AB31">
-        <f>IF(COUNT(B31:AA31)=0,"",SUM(B31:AA31))</f>
-        <v/>
-      </c>
-      <c r="AC31">
-        <f>COUNT(B31:AA31)</f>
-        <v/>
-      </c>
-      <c r="AD31">
-        <f>IF(OR(AB31="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB31,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB31,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z31="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z31,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z31,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2082,18 +2002,16 @@
       <c r="W32" s="5" t="n"/>
       <c r="X32" s="5" t="n"/>
       <c r="Y32" s="5" t="n"/>
-      <c r="Z32" s="5" t="n"/>
-      <c r="AA32" s="5" t="n"/>
+      <c r="Z32">
+        <f>IF(COUNT(B32:Y32)=0,"",SUM(B32:Y32))</f>
+        <v/>
+      </c>
+      <c r="AA32">
+        <f>COUNT(B32:Y32)</f>
+        <v/>
+      </c>
       <c r="AB32">
-        <f>IF(COUNT(B32:AA32)=0,"",SUM(B32:AA32))</f>
-        <v/>
-      </c>
-      <c r="AC32">
-        <f>COUNT(B32:AA32)</f>
-        <v/>
-      </c>
-      <c r="AD32">
-        <f>IF(OR(AB32="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB32,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB32,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z32="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z32,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z32,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2125,18 +2043,16 @@
       <c r="W33" s="5" t="n"/>
       <c r="X33" s="5" t="n"/>
       <c r="Y33" s="5" t="n"/>
-      <c r="Z33" s="5" t="n"/>
-      <c r="AA33" s="5" t="n"/>
+      <c r="Z33">
+        <f>IF(COUNT(B33:Y33)=0,"",SUM(B33:Y33))</f>
+        <v/>
+      </c>
+      <c r="AA33">
+        <f>COUNT(B33:Y33)</f>
+        <v/>
+      </c>
       <c r="AB33">
-        <f>IF(COUNT(B33:AA33)=0,"",SUM(B33:AA33))</f>
-        <v/>
-      </c>
-      <c r="AC33">
-        <f>COUNT(B33:AA33)</f>
-        <v/>
-      </c>
-      <c r="AD33">
-        <f>IF(OR(AB33="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB33,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB33,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z33="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z33,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z33,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2168,18 +2084,16 @@
       <c r="W34" s="5" t="n"/>
       <c r="X34" s="5" t="n"/>
       <c r="Y34" s="5" t="n"/>
-      <c r="Z34" s="5" t="n"/>
-      <c r="AA34" s="5" t="n"/>
+      <c r="Z34">
+        <f>IF(COUNT(B34:Y34)=0,"",SUM(B34:Y34))</f>
+        <v/>
+      </c>
+      <c r="AA34">
+        <f>COUNT(B34:Y34)</f>
+        <v/>
+      </c>
       <c r="AB34">
-        <f>IF(COUNT(B34:AA34)=0,"",SUM(B34:AA34))</f>
-        <v/>
-      </c>
-      <c r="AC34">
-        <f>COUNT(B34:AA34)</f>
-        <v/>
-      </c>
-      <c r="AD34">
-        <f>IF(OR(AB34="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB34,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB34,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z34="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z34,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z34,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2211,18 +2125,16 @@
       <c r="W35" s="5" t="n"/>
       <c r="X35" s="5" t="n"/>
       <c r="Y35" s="5" t="n"/>
-      <c r="Z35" s="5" t="n"/>
-      <c r="AA35" s="5" t="n"/>
+      <c r="Z35">
+        <f>IF(COUNT(B35:Y35)=0,"",SUM(B35:Y35))</f>
+        <v/>
+      </c>
+      <c r="AA35">
+        <f>COUNT(B35:Y35)</f>
+        <v/>
+      </c>
       <c r="AB35">
-        <f>IF(COUNT(B35:AA35)=0,"",SUM(B35:AA35))</f>
-        <v/>
-      </c>
-      <c r="AC35">
-        <f>COUNT(B35:AA35)</f>
-        <v/>
-      </c>
-      <c r="AD35">
-        <f>IF(OR(AB35="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB35,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB35,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z35="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z35,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z35,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2254,18 +2166,16 @@
       <c r="W36" s="5" t="n"/>
       <c r="X36" s="5" t="n"/>
       <c r="Y36" s="5" t="n"/>
-      <c r="Z36" s="5" t="n"/>
-      <c r="AA36" s="5" t="n"/>
+      <c r="Z36">
+        <f>IF(COUNT(B36:Y36)=0,"",SUM(B36:Y36))</f>
+        <v/>
+      </c>
+      <c r="AA36">
+        <f>COUNT(B36:Y36)</f>
+        <v/>
+      </c>
       <c r="AB36">
-        <f>IF(COUNT(B36:AA36)=0,"",SUM(B36:AA36))</f>
-        <v/>
-      </c>
-      <c r="AC36">
-        <f>COUNT(B36:AA36)</f>
-        <v/>
-      </c>
-      <c r="AD36">
-        <f>IF(OR(AB36="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB36,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB36,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z36="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z36,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z36,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2297,18 +2207,16 @@
       <c r="W37" s="5" t="n"/>
       <c r="X37" s="5" t="n"/>
       <c r="Y37" s="5" t="n"/>
-      <c r="Z37" s="5" t="n"/>
-      <c r="AA37" s="5" t="n"/>
+      <c r="Z37">
+        <f>IF(COUNT(B37:Y37)=0,"",SUM(B37:Y37))</f>
+        <v/>
+      </c>
+      <c r="AA37">
+        <f>COUNT(B37:Y37)</f>
+        <v/>
+      </c>
       <c r="AB37">
-        <f>IF(COUNT(B37:AA37)=0,"",SUM(B37:AA37))</f>
-        <v/>
-      </c>
-      <c r="AC37">
-        <f>COUNT(B37:AA37)</f>
-        <v/>
-      </c>
-      <c r="AD37">
-        <f>IF(OR(AB37="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB37,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB37,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z37="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z37,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z37,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2340,18 +2248,16 @@
       <c r="W38" s="5" t="n"/>
       <c r="X38" s="5" t="n"/>
       <c r="Y38" s="5" t="n"/>
-      <c r="Z38" s="5" t="n"/>
-      <c r="AA38" s="5" t="n"/>
+      <c r="Z38">
+        <f>IF(COUNT(B38:Y38)=0,"",SUM(B38:Y38))</f>
+        <v/>
+      </c>
+      <c r="AA38">
+        <f>COUNT(B38:Y38)</f>
+        <v/>
+      </c>
       <c r="AB38">
-        <f>IF(COUNT(B38:AA38)=0,"",SUM(B38:AA38))</f>
-        <v/>
-      </c>
-      <c r="AC38">
-        <f>COUNT(B38:AA38)</f>
-        <v/>
-      </c>
-      <c r="AD38">
-        <f>IF(OR(AB38="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB38,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB38,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z38="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z38,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z38,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2383,18 +2289,16 @@
       <c r="W39" s="5" t="n"/>
       <c r="X39" s="5" t="n"/>
       <c r="Y39" s="5" t="n"/>
-      <c r="Z39" s="5" t="n"/>
-      <c r="AA39" s="5" t="n"/>
+      <c r="Z39">
+        <f>IF(COUNT(B39:Y39)=0,"",SUM(B39:Y39))</f>
+        <v/>
+      </c>
+      <c r="AA39">
+        <f>COUNT(B39:Y39)</f>
+        <v/>
+      </c>
       <c r="AB39">
-        <f>IF(COUNT(B39:AA39)=0,"",SUM(B39:AA39))</f>
-        <v/>
-      </c>
-      <c r="AC39">
-        <f>COUNT(B39:AA39)</f>
-        <v/>
-      </c>
-      <c r="AD39">
-        <f>IF(OR(AB39="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB39,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB39,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z39="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z39,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z39,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2426,18 +2330,16 @@
       <c r="W40" s="5" t="n"/>
       <c r="X40" s="5" t="n"/>
       <c r="Y40" s="5" t="n"/>
-      <c r="Z40" s="5" t="n"/>
-      <c r="AA40" s="5" t="n"/>
+      <c r="Z40">
+        <f>IF(COUNT(B40:Y40)=0,"",SUM(B40:Y40))</f>
+        <v/>
+      </c>
+      <c r="AA40">
+        <f>COUNT(B40:Y40)</f>
+        <v/>
+      </c>
       <c r="AB40">
-        <f>IF(COUNT(B40:AA40)=0,"",SUM(B40:AA40))</f>
-        <v/>
-      </c>
-      <c r="AC40">
-        <f>COUNT(B40:AA40)</f>
-        <v/>
-      </c>
-      <c r="AD40">
-        <f>IF(OR(AB40="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB40,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB40,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z40="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z40,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z40,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2469,18 +2371,16 @@
       <c r="W41" s="5" t="n"/>
       <c r="X41" s="5" t="n"/>
       <c r="Y41" s="5" t="n"/>
-      <c r="Z41" s="5" t="n"/>
-      <c r="AA41" s="5" t="n"/>
+      <c r="Z41">
+        <f>IF(COUNT(B41:Y41)=0,"",SUM(B41:Y41))</f>
+        <v/>
+      </c>
+      <c r="AA41">
+        <f>COUNT(B41:Y41)</f>
+        <v/>
+      </c>
       <c r="AB41">
-        <f>IF(COUNT(B41:AA41)=0,"",SUM(B41:AA41))</f>
-        <v/>
-      </c>
-      <c r="AC41">
-        <f>COUNT(B41:AA41)</f>
-        <v/>
-      </c>
-      <c r="AD41">
-        <f>IF(OR(AB41="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB41,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB41,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z41="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z41,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z41,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2512,18 +2412,16 @@
       <c r="W42" s="5" t="n"/>
       <c r="X42" s="5" t="n"/>
       <c r="Y42" s="5" t="n"/>
-      <c r="Z42" s="5" t="n"/>
-      <c r="AA42" s="5" t="n"/>
+      <c r="Z42">
+        <f>IF(COUNT(B42:Y42)=0,"",SUM(B42:Y42))</f>
+        <v/>
+      </c>
+      <c r="AA42">
+        <f>COUNT(B42:Y42)</f>
+        <v/>
+      </c>
       <c r="AB42">
-        <f>IF(COUNT(B42:AA42)=0,"",SUM(B42:AA42))</f>
-        <v/>
-      </c>
-      <c r="AC42">
-        <f>COUNT(B42:AA42)</f>
-        <v/>
-      </c>
-      <c r="AD42">
-        <f>IF(OR(AB42="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB42,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB42,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z42="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z42,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z42,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2555,18 +2453,16 @@
       <c r="W43" s="5" t="n"/>
       <c r="X43" s="5" t="n"/>
       <c r="Y43" s="5" t="n"/>
-      <c r="Z43" s="5" t="n"/>
-      <c r="AA43" s="5" t="n"/>
+      <c r="Z43">
+        <f>IF(COUNT(B43:Y43)=0,"",SUM(B43:Y43))</f>
+        <v/>
+      </c>
+      <c r="AA43">
+        <f>COUNT(B43:Y43)</f>
+        <v/>
+      </c>
       <c r="AB43">
-        <f>IF(COUNT(B43:AA43)=0,"",SUM(B43:AA43))</f>
-        <v/>
-      </c>
-      <c r="AC43">
-        <f>COUNT(B43:AA43)</f>
-        <v/>
-      </c>
-      <c r="AD43">
-        <f>IF(OR(AB43="",COUNT($AB$5:$AB$43)&lt;3),"",IF(RANK(AB43,$AB$5:$AB$43,0)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"top",IF(RANK(AB43,$AB$5:$AB$43,1)&lt;=ROUND(COUNT($AB$5:$AB$43)/3,0),"bottom","middle")))</f>
+        <f>IF(OR(Z43="",COUNT($Z$5:$Z$43)&lt;3),"",IF(RANK(Z43,$Z$5:$Z$43,0)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"top",IF(RANK(Z43,$Z$5:$Z$43,1)&lt;=ROUND(COUNT($Z$5:$Z$43)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2581,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="13" max="13"/>
@@ -2706,11 +2602,11 @@
         <v/>
       </c>
       <c r="J5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!B$5:B$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!B$5:B$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!B$5:B$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!B$5:B$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!B$5:B$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!B$5:B$43)))</f>
         <v/>
       </c>
       <c r="K5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!B$5:B$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!B$5:B$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!B$5:B$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!B$5:B$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!B$5:B$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!B$5:B$43)))</f>
         <v/>
       </c>
       <c r="L5" s="6">
@@ -2750,7 +2646,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G6">
@@ -2766,11 +2662,11 @@
         <v/>
       </c>
       <c r="J6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!C$5:C$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!C$5:C$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!C$5:C$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!C$5:C$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!C$5:C$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!C$5:C$43)))</f>
         <v/>
       </c>
       <c r="K6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!C$5:C$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!C$5:C$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!C$5:C$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!C$5:C$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!C$5:C$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!C$5:C$43)))</f>
         <v/>
       </c>
       <c r="L6" s="6">
@@ -2826,11 +2722,11 @@
         <v/>
       </c>
       <c r="J7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!D$5:D$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!D$5:D$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!D$5:D$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!D$5:D$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!D$5:D$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!D$5:D$43)))</f>
         <v/>
       </c>
       <c r="K7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!D$5:D$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!D$5:D$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!D$5:D$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!D$5:D$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!D$5:D$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!D$5:D$43)))</f>
         <v/>
       </c>
       <c r="L7" s="6">
@@ -2886,11 +2782,11 @@
         <v/>
       </c>
       <c r="J8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!E$5:E$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!E$5:E$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!E$5:E$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!E$5:E$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!E$5:E$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!E$5:E$43)))</f>
         <v/>
       </c>
       <c r="K8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!E$5:E$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!E$5:E$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!E$5:E$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!E$5:E$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!E$5:E$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!E$5:E$43)))</f>
         <v/>
       </c>
       <c r="L8" s="6">
@@ -2946,11 +2842,11 @@
         <v/>
       </c>
       <c r="J9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!F$5:F$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!F$5:F$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!F$5:F$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!F$5:F$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!F$5:F$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!F$5:F$43)))</f>
         <v/>
       </c>
       <c r="K9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!F$5:F$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!F$5:F$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!F$5:F$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!F$5:F$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!F$5:F$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!F$5:F$43)))</f>
         <v/>
       </c>
       <c r="L9" s="6">
@@ -2980,7 +2876,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3006,11 +2902,11 @@
         <v/>
       </c>
       <c r="J10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!G$5:G$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!G$5:G$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!G$5:G$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!G$5:G$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!G$5:G$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!G$5:G$43)))</f>
         <v/>
       </c>
       <c r="K10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!G$5:G$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!G$5:G$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!G$5:G$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!G$5:G$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!G$5:G$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!G$5:G$43)))</f>
         <v/>
       </c>
       <c r="L10" s="6">
@@ -3040,7 +2936,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3066,11 +2962,11 @@
         <v/>
       </c>
       <c r="J11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!H$5:H$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!H$5:H$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!H$5:H$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!H$5:H$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!H$5:H$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!H$5:H$43)))</f>
         <v/>
       </c>
       <c r="K11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!H$5:H$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!H$5:H$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!H$5:H$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!H$5:H$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!H$5:H$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!H$5:H$43)))</f>
         <v/>
       </c>
       <c r="L11" s="6">
@@ -3110,7 +3006,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Call when p x 1,200 &gt; (1 - p) x 40, so p &gt; 40 / 1,240 = 1 / 31, about 0.032; the line moves down from 0.5 and recall leads.</t>
+          <t>Call when p x 1,200 &gt; (1 - p) x 40, so p &gt; 40 / 1,240 = 1 / 31, about 0.032 (1 in 30, 0.033, from one buyer paying for 30 calls, is accepted); the line moves down from 0.5 and recall leads.</t>
         </is>
       </c>
       <c r="G12">
@@ -3126,11 +3022,11 @@
         <v/>
       </c>
       <c r="J12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!I$5:I$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!I$5:I$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!I$5:I$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!I$5:I$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!I$5:I$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!I$5:I$43)))</f>
         <v/>
       </c>
       <c r="K12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!I$5:I$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!I$5:I$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!I$5:I$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!I$5:I$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!I$5:I$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!I$5:I$43)))</f>
         <v/>
       </c>
       <c r="L12" s="6">
@@ -3160,7 +3056,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3186,11 +3082,11 @@
         <v/>
       </c>
       <c r="J13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!J$5:J$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!J$5:J$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!J$5:J$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!J$5:J$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!J$5:J$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!J$5:J$43)))</f>
         <v/>
       </c>
       <c r="K13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!J$5:J$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!J$5:J$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!J$5:J$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!J$5:J$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!J$5:J$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!J$5:J$43)))</f>
         <v/>
       </c>
       <c r="L13" s="6">
@@ -3246,11 +3142,11 @@
         <v/>
       </c>
       <c r="J14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!K$5:K$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!K$5:K$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!K$5:K$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!K$5:K$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!K$5:K$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!K$5:K$43)))</f>
         <v/>
       </c>
       <c r="K14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!K$5:K$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!K$5:K$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!K$5:K$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!K$5:K$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!K$5:K$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!K$5:K$43)))</f>
         <v/>
       </c>
       <c r="L14" s="6">
@@ -3306,11 +3202,11 @@
         <v/>
       </c>
       <c r="J15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!L$5:L$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!L$5:L$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!L$5:L$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!L$5:L$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!L$5:L$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!L$5:L$43)))</f>
         <v/>
       </c>
       <c r="K15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!L$5:L$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!L$5:L$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!L$5:L$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!L$5:L$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!L$5:L$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!L$5:L$43)))</f>
         <v/>
       </c>
       <c r="L15" s="6">
@@ -3340,7 +3236,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3366,11 +3262,11 @@
         <v/>
       </c>
       <c r="J16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!M$5:M$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!M$5:M$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!M$5:M$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!M$5:M$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!M$5:M$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!M$5:M$43)))</f>
         <v/>
       </c>
       <c r="K16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!M$5:M$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!M$5:M$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!M$5:M$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!M$5:M$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!M$5:M$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!M$5:M$43)))</f>
         <v/>
       </c>
       <c r="L16" s="6">
@@ -3410,7 +3306,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>b, c, d</t>
+          <t>b, c</t>
         </is>
       </c>
       <c r="G17">
@@ -3426,11 +3322,11 @@
         <v/>
       </c>
       <c r="J17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!N$5:N$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!N$5:N$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!N$5:N$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!N$5:N$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!N$5:N$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!N$5:N$43)))</f>
         <v/>
       </c>
       <c r="K17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!N$5:N$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!N$5:N$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!N$5:N$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!N$5:N$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!N$5:N$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!N$5:N$43)))</f>
         <v/>
       </c>
       <c r="L17" s="6">
@@ -3486,11 +3382,11 @@
         <v/>
       </c>
       <c r="J18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!O$5:O$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!O$5:O$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!O$5:O$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!O$5:O$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!O$5:O$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!O$5:O$43)))</f>
         <v/>
       </c>
       <c r="K18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!O$5:O$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!O$5:O$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!O$5:O$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!O$5:O$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!O$5:O$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!O$5:O$43)))</f>
         <v/>
       </c>
       <c r="L18" s="6">
@@ -3520,7 +3416,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3546,11 +3442,11 @@
         <v/>
       </c>
       <c r="J19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!P$5:P$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!P$5:P$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!P$5:P$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!P$5:P$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!P$5:P$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!P$5:P$43)))</f>
         <v/>
       </c>
       <c r="K19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!P$5:P$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!P$5:P$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!P$5:P$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!P$5:P$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!P$5:P$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!P$5:P$43)))</f>
         <v/>
       </c>
       <c r="L19" s="6">
@@ -3606,11 +3502,11 @@
         <v/>
       </c>
       <c r="J20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!Q$5:Q$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!Q$5:Q$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!Q$5:Q$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!Q$5:Q$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!Q$5:Q$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!Q$5:Q$43)))</f>
         <v/>
       </c>
       <c r="K20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!Q$5:Q$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!Q$5:Q$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!Q$5:Q$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!Q$5:Q$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!Q$5:Q$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!Q$5:Q$43)))</f>
         <v/>
       </c>
       <c r="L20" s="6">
@@ -3640,7 +3536,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3666,11 +3562,11 @@
         <v/>
       </c>
       <c r="J21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!R$5:R$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!R$5:R$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!R$5:R$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!R$5:R$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!R$5:R$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!R$5:R$43)))</f>
         <v/>
       </c>
       <c r="K21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!R$5:R$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!R$5:R$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!R$5:R$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!R$5:R$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!R$5:R$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!R$5:R$43)))</f>
         <v/>
       </c>
       <c r="L21" s="6">
@@ -3726,11 +3622,11 @@
         <v/>
       </c>
       <c r="J22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!S$5:S$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!S$5:S$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!S$5:S$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!S$5:S$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!S$5:S$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!S$5:S$43)))</f>
         <v/>
       </c>
       <c r="K22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!S$5:S$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!S$5:S$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!S$5:S$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!S$5:S$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!S$5:S$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!S$5:S$43)))</f>
         <v/>
       </c>
       <c r="L22" s="6">
@@ -3786,11 +3682,11 @@
         <v/>
       </c>
       <c r="J23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!T$5:T$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!T$5:T$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!T$5:T$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!T$5:T$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!T$5:T$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!T$5:T$43)))</f>
         <v/>
       </c>
       <c r="K23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!T$5:T$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!T$5:T$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!T$5:T$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!T$5:T$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!T$5:T$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!T$5:T$43)))</f>
         <v/>
       </c>
       <c r="L23" s="6">
@@ -3830,7 +3726,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G24">
@@ -3846,11 +3742,11 @@
         <v/>
       </c>
       <c r="J24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!U$5:U$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!U$5:U$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!U$5:U$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!U$5:U$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!U$5:U$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!U$5:U$43)))</f>
         <v/>
       </c>
       <c r="K24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!U$5:U$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!U$5:U$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!U$5:U$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!U$5:U$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!U$5:U$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!U$5:U$43)))</f>
         <v/>
       </c>
       <c r="L24" s="6">
@@ -3871,21 +3767,21 @@
         <v>21</v>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fill in the blank</t>
+          <t>One correct option</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>[S]</t>
+          <t>[F]</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3906,11 +3802,11 @@
         <v/>
       </c>
       <c r="J25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!V$5:V$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!V$5:V$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!V$5:V$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!V$5:V$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!V$5:V$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!V$5:V$43)))</f>
         <v/>
       </c>
       <c r="K25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!V$5:V$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!V$5:V$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!V$5:V$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!V$5:V$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!V$5:V$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!V$5:V$43)))</f>
         <v/>
       </c>
       <c r="L25" s="6">
@@ -3931,11 +3827,11 @@
         <v>22</v>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fill in the blank</t>
+          <t>More than one correct</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3945,12 +3841,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[D]</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>b, c</t>
         </is>
       </c>
       <c r="G26">
@@ -3966,11 +3862,11 @@
         <v/>
       </c>
       <c r="J26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!W$5:W$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!W$5:W$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!W$5:W$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!W$5:W$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!W$5:W$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!W$5:W$43)))</f>
         <v/>
       </c>
       <c r="K26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!W$5:W$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!W$5:W$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!W$5:W$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!W$5:W$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!W$5:W$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!W$5:W$43)))</f>
         <v/>
       </c>
       <c r="L26" s="6">
@@ -4000,17 +3896,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>[F]</t>
+          <t>[D]</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G27">
@@ -4026,11 +3922,11 @@
         <v/>
       </c>
       <c r="J27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!X$5:X$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!X$5:X$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!X$5:X$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!X$5:X$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!X$5:X$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!X$5:X$43)))</f>
         <v/>
       </c>
       <c r="K27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!X$5:X$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!X$5:X$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!X$5:X$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!X$5:X$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!X$5:X$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!X$5:X$43)))</f>
         <v/>
       </c>
       <c r="L27" s="6">
@@ -4055,12 +3951,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>More than one correct</t>
+          <t>One correct option</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4070,7 +3966,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>b, c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G28">
@@ -4086,11 +3982,11 @@
         <v/>
       </c>
       <c r="J28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!Y$5:Y$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!Y$5:Y$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!Y$5:Y$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!Y$5:Y$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="top")*(Marks!Y$5:Y$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="top")*ISNUMBER(Marks!Y$5:Y$43)))</f>
         <v/>
       </c>
       <c r="K28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!Y$5:Y$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!Y$5:Y$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!Y$5:Y$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!Y$5:Y$43))=0,"",SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*(Marks!Y$5:Y$43=1))/SUMPRODUCT((Marks!$AB$5:$AB$43="bottom")*ISNUMBER(Marks!Y$5:Y$43)))</f>
         <v/>
       </c>
       <c r="L28" s="6">
@@ -4103,126 +3999,6 @@
       </c>
       <c r="N28">
         <f>IF(H28=0,"",I28+ROW()/1000000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" t="n">
-        <v>5</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>One correct option</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>[D]</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="G29">
-        <f>COUNTIF(Marks!Z$5:Z$43,1)</f>
-        <v/>
-      </c>
-      <c r="H29">
-        <f>COUNT(Marks!Z$5:Z$43)</f>
-        <v/>
-      </c>
-      <c r="I29" s="6">
-        <f>IF(H29=0,"",G29/H29)</f>
-        <v/>
-      </c>
-      <c r="J29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!Z$5:Z$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!Z$5:Z$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!Z$5:Z$43)))</f>
-        <v/>
-      </c>
-      <c r="K29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!Z$5:Z$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!Z$5:Z$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!Z$5:Z$43)))</f>
-        <v/>
-      </c>
-      <c r="L29" s="6">
-        <f>IF(OR(J29="",K29=""),"",J29-K29)</f>
-        <v/>
-      </c>
-      <c r="M29">
-        <f>IF(H29=0,"",IF(I29&lt;0.2,"Check the item: fewer than one in five got it right",IF(AND(L29&lt;&gt;"",N(L29)&lt;0),"Check the item: the bottom third beat the top third","")))</f>
-        <v/>
-      </c>
-      <c r="N29">
-        <f>IF(H29=0,"",I29+ROW()/1000000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>26</v>
-      </c>
-      <c r="B30" t="n">
-        <v>5</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>One correct option</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>[D]</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>d</t>
-        </is>
-      </c>
-      <c r="G30">
-        <f>COUNTIF(Marks!AA$5:AA$43,1)</f>
-        <v/>
-      </c>
-      <c r="H30">
-        <f>COUNT(Marks!AA$5:AA$43)</f>
-        <v/>
-      </c>
-      <c r="I30" s="6">
-        <f>IF(H30=0,"",G30/H30)</f>
-        <v/>
-      </c>
-      <c r="J30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!AA$5:AA$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="top")*(Marks!AA$5:AA$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="top")*ISNUMBER(Marks!AA$5:AA$43)))</f>
-        <v/>
-      </c>
-      <c r="K30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!AA$5:AA$43))=0,"",SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*(Marks!AA$5:AA$43=1))/SUMPRODUCT((Marks!$AD$5:$AD$43="bottom")*ISNUMBER(Marks!AA$5:AA$43)))</f>
-        <v/>
-      </c>
-      <c r="L30" s="6">
-        <f>IF(OR(J30="",K30=""),"",J30-K30)</f>
-        <v/>
-      </c>
-      <c r="M30">
-        <f>IF(H30=0,"",IF(I30&lt;0.2,"Check the item: fewer than one in five got it right",IF(AND(L30&lt;&gt;"",N(L30)&lt;0),"Check the item: the bottom third beat the top third","")))</f>
-        <v/>
-      </c>
-      <c r="N30">
-        <f>IF(H30=0,"",I30+ROW()/1000000)</f>
         <v/>
       </c>
     </row>
@@ -4237,7 +4013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="6" max="6"/>
@@ -4252,7 +4028,7 @@
     </row>
     <row r="2">
       <c r="B2">
-        <f>IF(SUM(Items!H5:H30)=0,"No marks entered yet.","Most-missed first: take the items from the top.")</f>
+        <f>IF(SUM(Items!H5:H28)=0,"No marks entered yet.","Most-missed first: take the items from the top.")</f>
         <v/>
       </c>
     </row>
@@ -4293,23 +4069,23 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A5,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A5),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A5,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A5),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>IF(B5="","",INDEX(Items!$I$5:$I$30,MATCH(B5,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B5="","",INDEX(Items!$I$5:$I$28,MATCH(B5,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D5">
-        <f>IF(B5="","",INDEX(Items!$B$5:$B$30,MATCH(B5,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B5="","",INDEX(Items!$B$5:$B$28,MATCH(B5,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E5">
-        <f>IF(B5="","",INDEX(Items!$E$5:$E$30,MATCH(B5,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B5="","",INDEX(Items!$E$5:$E$28,MATCH(B5,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F5">
-        <f>IF(B5="","",INDEX(Items!$M$5:$M$30,MATCH(B5,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B5="","",INDEX(Items!$M$5:$M$28,MATCH(B5,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4318,23 +4094,23 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A6,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A6),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A6,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A6),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>IF(B6="","",INDEX(Items!$I$5:$I$30,MATCH(B6,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B6="","",INDEX(Items!$I$5:$I$28,MATCH(B6,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D6">
-        <f>IF(B6="","",INDEX(Items!$B$5:$B$30,MATCH(B6,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B6="","",INDEX(Items!$B$5:$B$28,MATCH(B6,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E6">
-        <f>IF(B6="","",INDEX(Items!$E$5:$E$30,MATCH(B6,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B6="","",INDEX(Items!$E$5:$E$28,MATCH(B6,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F6">
-        <f>IF(B6="","",INDEX(Items!$M$5:$M$30,MATCH(B6,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B6="","",INDEX(Items!$M$5:$M$28,MATCH(B6,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4343,23 +4119,23 @@
         <v>3</v>
       </c>
       <c r="B7">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A7,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A7),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A7,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A7),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>IF(B7="","",INDEX(Items!$I$5:$I$30,MATCH(B7,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B7="","",INDEX(Items!$I$5:$I$28,MATCH(B7,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D7">
-        <f>IF(B7="","",INDEX(Items!$B$5:$B$30,MATCH(B7,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B7="","",INDEX(Items!$B$5:$B$28,MATCH(B7,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E7">
-        <f>IF(B7="","",INDEX(Items!$E$5:$E$30,MATCH(B7,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B7="","",INDEX(Items!$E$5:$E$28,MATCH(B7,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F7">
-        <f>IF(B7="","",INDEX(Items!$M$5:$M$30,MATCH(B7,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B7="","",INDEX(Items!$M$5:$M$28,MATCH(B7,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4368,23 +4144,23 @@
         <v>4</v>
       </c>
       <c r="B8">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A8,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A8),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A8,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A8),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>IF(B8="","",INDEX(Items!$I$5:$I$30,MATCH(B8,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B8="","",INDEX(Items!$I$5:$I$28,MATCH(B8,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D8">
-        <f>IF(B8="","",INDEX(Items!$B$5:$B$30,MATCH(B8,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B8="","",INDEX(Items!$B$5:$B$28,MATCH(B8,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E8">
-        <f>IF(B8="","",INDEX(Items!$E$5:$E$30,MATCH(B8,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B8="","",INDEX(Items!$E$5:$E$28,MATCH(B8,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F8">
-        <f>IF(B8="","",INDEX(Items!$M$5:$M$30,MATCH(B8,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B8="","",INDEX(Items!$M$5:$M$28,MATCH(B8,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4393,23 +4169,23 @@
         <v>5</v>
       </c>
       <c r="B9">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A9,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A9),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A9,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A9),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>IF(B9="","",INDEX(Items!$I$5:$I$30,MATCH(B9,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B9="","",INDEX(Items!$I$5:$I$28,MATCH(B9,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D9">
-        <f>IF(B9="","",INDEX(Items!$B$5:$B$30,MATCH(B9,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B9="","",INDEX(Items!$B$5:$B$28,MATCH(B9,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E9">
-        <f>IF(B9="","",INDEX(Items!$E$5:$E$30,MATCH(B9,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B9="","",INDEX(Items!$E$5:$E$28,MATCH(B9,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F9">
-        <f>IF(B9="","",INDEX(Items!$M$5:$M$30,MATCH(B9,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B9="","",INDEX(Items!$M$5:$M$28,MATCH(B9,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4418,23 +4194,23 @@
         <v>6</v>
       </c>
       <c r="B10">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A10,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A10),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A10,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A10),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C10" s="6">
-        <f>IF(B10="","",INDEX(Items!$I$5:$I$30,MATCH(B10,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B10="","",INDEX(Items!$I$5:$I$28,MATCH(B10,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D10">
-        <f>IF(B10="","",INDEX(Items!$B$5:$B$30,MATCH(B10,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B10="","",INDEX(Items!$B$5:$B$28,MATCH(B10,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E10">
-        <f>IF(B10="","",INDEX(Items!$E$5:$E$30,MATCH(B10,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B10="","",INDEX(Items!$E$5:$E$28,MATCH(B10,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F10">
-        <f>IF(B10="","",INDEX(Items!$M$5:$M$30,MATCH(B10,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B10="","",INDEX(Items!$M$5:$M$28,MATCH(B10,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4443,23 +4219,23 @@
         <v>7</v>
       </c>
       <c r="B11">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A11,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A11),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A11,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A11),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C11" s="6">
-        <f>IF(B11="","",INDEX(Items!$I$5:$I$30,MATCH(B11,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B11="","",INDEX(Items!$I$5:$I$28,MATCH(B11,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D11">
-        <f>IF(B11="","",INDEX(Items!$B$5:$B$30,MATCH(B11,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B11="","",INDEX(Items!$B$5:$B$28,MATCH(B11,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E11">
-        <f>IF(B11="","",INDEX(Items!$E$5:$E$30,MATCH(B11,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B11="","",INDEX(Items!$E$5:$E$28,MATCH(B11,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F11">
-        <f>IF(B11="","",INDEX(Items!$M$5:$M$30,MATCH(B11,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B11="","",INDEX(Items!$M$5:$M$28,MATCH(B11,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4468,23 +4244,23 @@
         <v>8</v>
       </c>
       <c r="B12">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A12,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A12),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A12,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A12),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C12" s="6">
-        <f>IF(B12="","",INDEX(Items!$I$5:$I$30,MATCH(B12,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B12="","",INDEX(Items!$I$5:$I$28,MATCH(B12,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D12">
-        <f>IF(B12="","",INDEX(Items!$B$5:$B$30,MATCH(B12,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B12="","",INDEX(Items!$B$5:$B$28,MATCH(B12,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E12">
-        <f>IF(B12="","",INDEX(Items!$E$5:$E$30,MATCH(B12,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B12="","",INDEX(Items!$E$5:$E$28,MATCH(B12,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F12">
-        <f>IF(B12="","",INDEX(Items!$M$5:$M$30,MATCH(B12,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B12="","",INDEX(Items!$M$5:$M$28,MATCH(B12,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4493,23 +4269,23 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A13,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A13),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A13,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A13),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C13" s="6">
-        <f>IF(B13="","",INDEX(Items!$I$5:$I$30,MATCH(B13,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B13="","",INDEX(Items!$I$5:$I$28,MATCH(B13,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D13">
-        <f>IF(B13="","",INDEX(Items!$B$5:$B$30,MATCH(B13,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B13="","",INDEX(Items!$B$5:$B$28,MATCH(B13,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E13">
-        <f>IF(B13="","",INDEX(Items!$E$5:$E$30,MATCH(B13,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B13="","",INDEX(Items!$E$5:$E$28,MATCH(B13,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F13">
-        <f>IF(B13="","",INDEX(Items!$M$5:$M$30,MATCH(B13,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B13="","",INDEX(Items!$M$5:$M$28,MATCH(B13,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4518,23 +4294,23 @@
         <v>10</v>
       </c>
       <c r="B14">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A14,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A14),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A14,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A14),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C14" s="6">
-        <f>IF(B14="","",INDEX(Items!$I$5:$I$30,MATCH(B14,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B14="","",INDEX(Items!$I$5:$I$28,MATCH(B14,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D14">
-        <f>IF(B14="","",INDEX(Items!$B$5:$B$30,MATCH(B14,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B14="","",INDEX(Items!$B$5:$B$28,MATCH(B14,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E14">
-        <f>IF(B14="","",INDEX(Items!$E$5:$E$30,MATCH(B14,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B14="","",INDEX(Items!$E$5:$E$28,MATCH(B14,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F14">
-        <f>IF(B14="","",INDEX(Items!$M$5:$M$30,MATCH(B14,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B14="","",INDEX(Items!$M$5:$M$28,MATCH(B14,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4543,23 +4319,23 @@
         <v>11</v>
       </c>
       <c r="B15">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A15,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A15),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A15,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A15),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C15" s="6">
-        <f>IF(B15="","",INDEX(Items!$I$5:$I$30,MATCH(B15,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B15="","",INDEX(Items!$I$5:$I$28,MATCH(B15,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D15">
-        <f>IF(B15="","",INDEX(Items!$B$5:$B$30,MATCH(B15,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B15="","",INDEX(Items!$B$5:$B$28,MATCH(B15,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E15">
-        <f>IF(B15="","",INDEX(Items!$E$5:$E$30,MATCH(B15,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B15="","",INDEX(Items!$E$5:$E$28,MATCH(B15,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F15">
-        <f>IF(B15="","",INDEX(Items!$M$5:$M$30,MATCH(B15,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B15="","",INDEX(Items!$M$5:$M$28,MATCH(B15,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4568,23 +4344,23 @@
         <v>12</v>
       </c>
       <c r="B16">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A16,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A16),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A16,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A16),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C16" s="6">
-        <f>IF(B16="","",INDEX(Items!$I$5:$I$30,MATCH(B16,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B16="","",INDEX(Items!$I$5:$I$28,MATCH(B16,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D16">
-        <f>IF(B16="","",INDEX(Items!$B$5:$B$30,MATCH(B16,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B16="","",INDEX(Items!$B$5:$B$28,MATCH(B16,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E16">
-        <f>IF(B16="","",INDEX(Items!$E$5:$E$30,MATCH(B16,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B16="","",INDEX(Items!$E$5:$E$28,MATCH(B16,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F16">
-        <f>IF(B16="","",INDEX(Items!$M$5:$M$30,MATCH(B16,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B16="","",INDEX(Items!$M$5:$M$28,MATCH(B16,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4593,23 +4369,23 @@
         <v>13</v>
       </c>
       <c r="B17">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A17,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A17),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A17,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A17),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C17" s="6">
-        <f>IF(B17="","",INDEX(Items!$I$5:$I$30,MATCH(B17,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B17="","",INDEX(Items!$I$5:$I$28,MATCH(B17,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D17">
-        <f>IF(B17="","",INDEX(Items!$B$5:$B$30,MATCH(B17,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B17="","",INDEX(Items!$B$5:$B$28,MATCH(B17,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E17">
-        <f>IF(B17="","",INDEX(Items!$E$5:$E$30,MATCH(B17,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B17="","",INDEX(Items!$E$5:$E$28,MATCH(B17,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F17">
-        <f>IF(B17="","",INDEX(Items!$M$5:$M$30,MATCH(B17,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B17="","",INDEX(Items!$M$5:$M$28,MATCH(B17,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4618,23 +4394,23 @@
         <v>14</v>
       </c>
       <c r="B18">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A18,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A18),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A18,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A18),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C18" s="6">
-        <f>IF(B18="","",INDEX(Items!$I$5:$I$30,MATCH(B18,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B18="","",INDEX(Items!$I$5:$I$28,MATCH(B18,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D18">
-        <f>IF(B18="","",INDEX(Items!$B$5:$B$30,MATCH(B18,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B18="","",INDEX(Items!$B$5:$B$28,MATCH(B18,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E18">
-        <f>IF(B18="","",INDEX(Items!$E$5:$E$30,MATCH(B18,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B18="","",INDEX(Items!$E$5:$E$28,MATCH(B18,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F18">
-        <f>IF(B18="","",INDEX(Items!$M$5:$M$30,MATCH(B18,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B18="","",INDEX(Items!$M$5:$M$28,MATCH(B18,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4643,23 +4419,23 @@
         <v>15</v>
       </c>
       <c r="B19">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A19,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A19),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A19,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A19),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C19" s="6">
-        <f>IF(B19="","",INDEX(Items!$I$5:$I$30,MATCH(B19,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B19="","",INDEX(Items!$I$5:$I$28,MATCH(B19,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D19">
-        <f>IF(B19="","",INDEX(Items!$B$5:$B$30,MATCH(B19,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B19="","",INDEX(Items!$B$5:$B$28,MATCH(B19,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E19">
-        <f>IF(B19="","",INDEX(Items!$E$5:$E$30,MATCH(B19,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B19="","",INDEX(Items!$E$5:$E$28,MATCH(B19,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F19">
-        <f>IF(B19="","",INDEX(Items!$M$5:$M$30,MATCH(B19,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B19="","",INDEX(Items!$M$5:$M$28,MATCH(B19,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4668,23 +4444,23 @@
         <v>16</v>
       </c>
       <c r="B20">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A20,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A20),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A20,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A20),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C20" s="6">
-        <f>IF(B20="","",INDEX(Items!$I$5:$I$30,MATCH(B20,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B20="","",INDEX(Items!$I$5:$I$28,MATCH(B20,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D20">
-        <f>IF(B20="","",INDEX(Items!$B$5:$B$30,MATCH(B20,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B20="","",INDEX(Items!$B$5:$B$28,MATCH(B20,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E20">
-        <f>IF(B20="","",INDEX(Items!$E$5:$E$30,MATCH(B20,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B20="","",INDEX(Items!$E$5:$E$28,MATCH(B20,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F20">
-        <f>IF(B20="","",INDEX(Items!$M$5:$M$30,MATCH(B20,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B20="","",INDEX(Items!$M$5:$M$28,MATCH(B20,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4693,23 +4469,23 @@
         <v>17</v>
       </c>
       <c r="B21">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A21,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A21),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A21,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A21),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C21" s="6">
-        <f>IF(B21="","",INDEX(Items!$I$5:$I$30,MATCH(B21,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B21="","",INDEX(Items!$I$5:$I$28,MATCH(B21,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D21">
-        <f>IF(B21="","",INDEX(Items!$B$5:$B$30,MATCH(B21,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B21="","",INDEX(Items!$B$5:$B$28,MATCH(B21,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E21">
-        <f>IF(B21="","",INDEX(Items!$E$5:$E$30,MATCH(B21,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B21="","",INDEX(Items!$E$5:$E$28,MATCH(B21,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F21">
-        <f>IF(B21="","",INDEX(Items!$M$5:$M$30,MATCH(B21,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B21="","",INDEX(Items!$M$5:$M$28,MATCH(B21,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4718,23 +4494,23 @@
         <v>18</v>
       </c>
       <c r="B22">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A22,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A22),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A22,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A22),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C22" s="6">
-        <f>IF(B22="","",INDEX(Items!$I$5:$I$30,MATCH(B22,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B22="","",INDEX(Items!$I$5:$I$28,MATCH(B22,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D22">
-        <f>IF(B22="","",INDEX(Items!$B$5:$B$30,MATCH(B22,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B22="","",INDEX(Items!$B$5:$B$28,MATCH(B22,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E22">
-        <f>IF(B22="","",INDEX(Items!$E$5:$E$30,MATCH(B22,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B22="","",INDEX(Items!$E$5:$E$28,MATCH(B22,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F22">
-        <f>IF(B22="","",INDEX(Items!$M$5:$M$30,MATCH(B22,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B22="","",INDEX(Items!$M$5:$M$28,MATCH(B22,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4743,23 +4519,23 @@
         <v>19</v>
       </c>
       <c r="B23">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A23,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A23),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A23,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A23),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C23" s="6">
-        <f>IF(B23="","",INDEX(Items!$I$5:$I$30,MATCH(B23,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B23="","",INDEX(Items!$I$5:$I$28,MATCH(B23,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D23">
-        <f>IF(B23="","",INDEX(Items!$B$5:$B$30,MATCH(B23,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B23="","",INDEX(Items!$B$5:$B$28,MATCH(B23,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E23">
-        <f>IF(B23="","",INDEX(Items!$E$5:$E$30,MATCH(B23,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B23="","",INDEX(Items!$E$5:$E$28,MATCH(B23,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F23">
-        <f>IF(B23="","",INDEX(Items!$M$5:$M$30,MATCH(B23,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B23="","",INDEX(Items!$M$5:$M$28,MATCH(B23,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4768,23 +4544,23 @@
         <v>20</v>
       </c>
       <c r="B24">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A24,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A24),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A24,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A24),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C24" s="6">
-        <f>IF(B24="","",INDEX(Items!$I$5:$I$30,MATCH(B24,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B24="","",INDEX(Items!$I$5:$I$28,MATCH(B24,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D24">
-        <f>IF(B24="","",INDEX(Items!$B$5:$B$30,MATCH(B24,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B24="","",INDEX(Items!$B$5:$B$28,MATCH(B24,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E24">
-        <f>IF(B24="","",INDEX(Items!$E$5:$E$30,MATCH(B24,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B24="","",INDEX(Items!$E$5:$E$28,MATCH(B24,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F24">
-        <f>IF(B24="","",INDEX(Items!$M$5:$M$30,MATCH(B24,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B24="","",INDEX(Items!$M$5:$M$28,MATCH(B24,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4793,23 +4569,23 @@
         <v>21</v>
       </c>
       <c r="B25">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A25,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A25),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A25,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A25),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C25" s="6">
-        <f>IF(B25="","",INDEX(Items!$I$5:$I$30,MATCH(B25,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B25="","",INDEX(Items!$I$5:$I$28,MATCH(B25,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D25">
-        <f>IF(B25="","",INDEX(Items!$B$5:$B$30,MATCH(B25,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B25="","",INDEX(Items!$B$5:$B$28,MATCH(B25,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E25">
-        <f>IF(B25="","",INDEX(Items!$E$5:$E$30,MATCH(B25,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B25="","",INDEX(Items!$E$5:$E$28,MATCH(B25,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F25">
-        <f>IF(B25="","",INDEX(Items!$M$5:$M$30,MATCH(B25,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B25="","",INDEX(Items!$M$5:$M$28,MATCH(B25,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4818,23 +4594,23 @@
         <v>22</v>
       </c>
       <c r="B26">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A26,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A26),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A26,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A26),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C26" s="6">
-        <f>IF(B26="","",INDEX(Items!$I$5:$I$30,MATCH(B26,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B26="","",INDEX(Items!$I$5:$I$28,MATCH(B26,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D26">
-        <f>IF(B26="","",INDEX(Items!$B$5:$B$30,MATCH(B26,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B26="","",INDEX(Items!$B$5:$B$28,MATCH(B26,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E26">
-        <f>IF(B26="","",INDEX(Items!$E$5:$E$30,MATCH(B26,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B26="","",INDEX(Items!$E$5:$E$28,MATCH(B26,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F26">
-        <f>IF(B26="","",INDEX(Items!$M$5:$M$30,MATCH(B26,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B26="","",INDEX(Items!$M$5:$M$28,MATCH(B26,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4843,23 +4619,23 @@
         <v>23</v>
       </c>
       <c r="B27">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A27,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A27),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A27,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A27),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C27" s="6">
-        <f>IF(B27="","",INDEX(Items!$I$5:$I$30,MATCH(B27,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B27="","",INDEX(Items!$I$5:$I$28,MATCH(B27,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D27">
-        <f>IF(B27="","",INDEX(Items!$B$5:$B$30,MATCH(B27,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B27="","",INDEX(Items!$B$5:$B$28,MATCH(B27,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E27">
-        <f>IF(B27="","",INDEX(Items!$E$5:$E$30,MATCH(B27,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B27="","",INDEX(Items!$E$5:$E$28,MATCH(B27,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F27">
-        <f>IF(B27="","",INDEX(Items!$M$5:$M$30,MATCH(B27,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B27="","",INDEX(Items!$M$5:$M$28,MATCH(B27,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4868,73 +4644,23 @@
         <v>24</v>
       </c>
       <c r="B28">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A28,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A28),Items!$N$5:$N$30,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$28)&lt;A28,"",INDEX(Items!$A$5:$A$28,MATCH(SMALL(Items!$N$5:$N$28,A28),Items!$N$5:$N$28,0)))</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>IF(B28="","",INDEX(Items!$I$5:$I$30,MATCH(B28,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B28="","",INDEX(Items!$I$5:$I$28,MATCH(B28,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="D28">
-        <f>IF(B28="","",INDEX(Items!$B$5:$B$30,MATCH(B28,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B28="","",INDEX(Items!$B$5:$B$28,MATCH(B28,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="E28">
-        <f>IF(B28="","",INDEX(Items!$E$5:$E$30,MATCH(B28,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B28="","",INDEX(Items!$E$5:$E$28,MATCH(B28,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
       <c r="F28">
-        <f>IF(B28="","",INDEX(Items!$M$5:$M$30,MATCH(B28,Items!$A$5:$A$30,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A29,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A29),Items!$N$5:$N$30,0)))</f>
-        <v/>
-      </c>
-      <c r="C29" s="6">
-        <f>IF(B29="","",INDEX(Items!$I$5:$I$30,MATCH(B29,Items!$A$5:$A$30,0)))</f>
-        <v/>
-      </c>
-      <c r="D29">
-        <f>IF(B29="","",INDEX(Items!$B$5:$B$30,MATCH(B29,Items!$A$5:$A$30,0)))</f>
-        <v/>
-      </c>
-      <c r="E29">
-        <f>IF(B29="","",INDEX(Items!$E$5:$E$30,MATCH(B29,Items!$A$5:$A$30,0)))</f>
-        <v/>
-      </c>
-      <c r="F29">
-        <f>IF(B29="","",INDEX(Items!$M$5:$M$30,MATCH(B29,Items!$A$5:$A$30,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>26</v>
-      </c>
-      <c r="B30">
-        <f>IF(COUNT(Items!$N$5:$N$30)&lt;A30,"",INDEX(Items!$A$5:$A$30,MATCH(SMALL(Items!$N$5:$N$30,A30),Items!$N$5:$N$30,0)))</f>
-        <v/>
-      </c>
-      <c r="C30" s="6">
-        <f>IF(B30="","",INDEX(Items!$I$5:$I$30,MATCH(B30,Items!$A$5:$A$30,0)))</f>
-        <v/>
-      </c>
-      <c r="D30">
-        <f>IF(B30="","",INDEX(Items!$B$5:$B$30,MATCH(B30,Items!$A$5:$A$30,0)))</f>
-        <v/>
-      </c>
-      <c r="E30">
-        <f>IF(B30="","",INDEX(Items!$E$5:$E$30,MATCH(B30,Items!$A$5:$A$30,0)))</f>
-        <v/>
-      </c>
-      <c r="F30">
-        <f>IF(B30="","",INDEX(Items!$M$5:$M$30,MATCH(B30,Items!$A$5:$A$30,0)))</f>
+        <f>IF(B28="","",INDEX(Items!$M$5:$M$28,MATCH(B28,Items!$A$5:$A$28,0)))</f>
         <v/>
       </c>
     </row>
@@ -4996,11 +4722,11 @@
         </is>
       </c>
       <c r="C5">
-        <f>COUNTIF(Items!$E$5:$E$30,A5)</f>
+        <f>COUNTIF(Items!$E$5:$E$28,A5)</f>
         <v/>
       </c>
       <c r="D5" s="6">
-        <f>IF(SUMPRODUCT((Items!$E$5:$E$30=A5)*Items!$H$5:$H$30)=0,"",SUMPRODUCT((Items!$E$5:$E$30=A5)*Items!$G$5:$G$30)/SUMPRODUCT((Items!$E$5:$E$30=A5)*Items!$H$5:$H$30))</f>
+        <f>IF(SUMPRODUCT((Items!$E$5:$E$28=A5)*Items!$H$5:$H$28)=0,"",SUMPRODUCT((Items!$E$5:$E$28=A5)*Items!$G$5:$G$28)/SUMPRODUCT((Items!$E$5:$E$28=A5)*Items!$H$5:$H$28))</f>
         <v/>
       </c>
     </row>
@@ -5016,11 +4742,11 @@
         </is>
       </c>
       <c r="C6">
-        <f>COUNTIF(Items!$E$5:$E$30,A6)</f>
+        <f>COUNTIF(Items!$E$5:$E$28,A6)</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>IF(SUMPRODUCT((Items!$E$5:$E$30=A6)*Items!$H$5:$H$30)=0,"",SUMPRODUCT((Items!$E$5:$E$30=A6)*Items!$G$5:$G$30)/SUMPRODUCT((Items!$E$5:$E$30=A6)*Items!$H$5:$H$30))</f>
+        <f>IF(SUMPRODUCT((Items!$E$5:$E$28=A6)*Items!$H$5:$H$28)=0,"",SUMPRODUCT((Items!$E$5:$E$28=A6)*Items!$G$5:$G$28)/SUMPRODUCT((Items!$E$5:$E$28=A6)*Items!$H$5:$H$28))</f>
         <v/>
       </c>
     </row>
@@ -5036,11 +4762,11 @@
         </is>
       </c>
       <c r="C7">
-        <f>COUNTIF(Items!$E$5:$E$30,A7)</f>
+        <f>COUNTIF(Items!$E$5:$E$28,A7)</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>IF(SUMPRODUCT((Items!$E$5:$E$30=A7)*Items!$H$5:$H$30)=0,"",SUMPRODUCT((Items!$E$5:$E$30=A7)*Items!$G$5:$G$30)/SUMPRODUCT((Items!$E$5:$E$30=A7)*Items!$H$5:$H$30))</f>
+        <f>IF(SUMPRODUCT((Items!$E$5:$E$28=A7)*Items!$H$5:$H$28)=0,"",SUMPRODUCT((Items!$E$5:$E$28=A7)*Items!$G$5:$G$28)/SUMPRODUCT((Items!$E$5:$E$28=A7)*Items!$H$5:$H$28))</f>
         <v/>
       </c>
     </row>
@@ -5054,11 +4780,11 @@
         </is>
       </c>
       <c r="C8">
-        <f>COUNTIF(Items!$B$5:$B$30,A8)</f>
+        <f>COUNTIF(Items!$B$5:$B$28,A8)</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$30=A8)*Items!$H$5:$H$30)=0,"",SUMPRODUCT((Items!$B$5:$B$30=A8)*Items!$G$5:$G$30)/SUMPRODUCT((Items!$B$5:$B$30=A8)*Items!$H$5:$H$30))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$28=A8)*Items!$H$5:$H$28)=0,"",SUMPRODUCT((Items!$B$5:$B$28=A8)*Items!$G$5:$G$28)/SUMPRODUCT((Items!$B$5:$B$28=A8)*Items!$H$5:$H$28))</f>
         <v/>
       </c>
     </row>
@@ -5072,11 +4798,11 @@
         </is>
       </c>
       <c r="C9">
-        <f>COUNTIF(Items!$B$5:$B$30,A9)</f>
+        <f>COUNTIF(Items!$B$5:$B$28,A9)</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$30=A9)*Items!$H$5:$H$30)=0,"",SUMPRODUCT((Items!$B$5:$B$30=A9)*Items!$G$5:$G$30)/SUMPRODUCT((Items!$B$5:$B$30=A9)*Items!$H$5:$H$30))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$28=A9)*Items!$H$5:$H$28)=0,"",SUMPRODUCT((Items!$B$5:$B$28=A9)*Items!$G$5:$G$28)/SUMPRODUCT((Items!$B$5:$B$28=A9)*Items!$H$5:$H$28))</f>
         <v/>
       </c>
     </row>
@@ -5090,11 +4816,11 @@
         </is>
       </c>
       <c r="C10">
-        <f>COUNTIF(Items!$B$5:$B$30,A10)</f>
+        <f>COUNTIF(Items!$B$5:$B$28,A10)</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$30=A10)*Items!$H$5:$H$30)=0,"",SUMPRODUCT((Items!$B$5:$B$30=A10)*Items!$G$5:$G$30)/SUMPRODUCT((Items!$B$5:$B$30=A10)*Items!$H$5:$H$30))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$28=A10)*Items!$H$5:$H$28)=0,"",SUMPRODUCT((Items!$B$5:$B$28=A10)*Items!$G$5:$G$28)/SUMPRODUCT((Items!$B$5:$B$28=A10)*Items!$H$5:$H$28))</f>
         <v/>
       </c>
     </row>
@@ -5108,11 +4834,11 @@
         </is>
       </c>
       <c r="C11">
-        <f>COUNTIF(Items!$B$5:$B$30,A11)</f>
+        <f>COUNTIF(Items!$B$5:$B$28,A11)</f>
         <v/>
       </c>
       <c r="D11" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$30=A11)*Items!$H$5:$H$30)=0,"",SUMPRODUCT((Items!$B$5:$B$30=A11)*Items!$G$5:$G$30)/SUMPRODUCT((Items!$B$5:$B$30=A11)*Items!$H$5:$H$30))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$28=A11)*Items!$H$5:$H$28)=0,"",SUMPRODUCT((Items!$B$5:$B$28=A11)*Items!$G$5:$G$28)/SUMPRODUCT((Items!$B$5:$B$28=A11)*Items!$H$5:$H$28))</f>
         <v/>
       </c>
     </row>
@@ -5126,11 +4852,11 @@
         </is>
       </c>
       <c r="C12">
-        <f>COUNTIF(Items!$B$5:$B$30,A12)</f>
+        <f>COUNTIF(Items!$B$5:$B$28,A12)</f>
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$30=A12)*Items!$H$5:$H$30)=0,"",SUMPRODUCT((Items!$B$5:$B$30=A12)*Items!$G$5:$G$30)/SUMPRODUCT((Items!$B$5:$B$30=A12)*Items!$H$5:$H$30))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$28=A12)*Items!$H$5:$H$28)=0,"",SUMPRODUCT((Items!$B$5:$B$28=A12)*Items!$G$5:$G$28)/SUMPRODUCT((Items!$B$5:$B$28=A12)*Items!$H$5:$H$28))</f>
         <v/>
       </c>
     </row>
@@ -5182,15 +4908,15 @@
         <v>1</v>
       </c>
       <c r="B5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$5:$AA$5))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$5:$AA$5=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$5:$AA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$5:$Y$5))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$5:$Y$5=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$5:$Y$5)))</f>
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$5:$AA$5))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$5:$AA$5=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$5:$AA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$5:$Y$5))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$5:$Y$5=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$5:$Y$5)))</f>
         <v/>
       </c>
       <c r="D5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$5:$AA$5))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$5:$AA$5=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$5:$AA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$5:$Y$5))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$5:$Y$5=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$5:$Y$5)))</f>
         <v/>
       </c>
     </row>
@@ -5199,15 +4925,15 @@
         <v>2</v>
       </c>
       <c r="B6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$6:$AA$6))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$6:$AA$6=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$6:$AA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$6:$Y$6))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$6:$Y$6=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$6:$Y$6)))</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$6:$AA$6))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$6:$AA$6=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$6:$AA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$6:$Y$6))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$6:$Y$6=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$6:$Y$6)))</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$6:$AA$6))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$6:$AA$6=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$6:$AA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$6:$Y$6))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$6:$Y$6=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$6:$Y$6)))</f>
         <v/>
       </c>
     </row>
@@ -5216,15 +4942,15 @@
         <v>3</v>
       </c>
       <c r="B7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$7:$AA$7))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$7:$AA$7=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$7:$AA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$7:$Y$7))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$7:$Y$7=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$7:$Y$7)))</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$7:$AA$7))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$7:$AA$7=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$7:$AA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$7:$Y$7))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$7:$Y$7=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$7:$Y$7)))</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$7:$AA$7))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$7:$AA$7=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$7:$AA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$7:$Y$7))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$7:$Y$7=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$7:$Y$7)))</f>
         <v/>
       </c>
     </row>
@@ -5233,15 +4959,15 @@
         <v>4</v>
       </c>
       <c r="B8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$8:$AA$8))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$8:$AA$8=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$8:$AA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$8:$Y$8))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$8:$Y$8=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$8:$Y$8)))</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$8:$AA$8))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$8:$AA$8=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$8:$AA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$8:$Y$8))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$8:$Y$8=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$8:$Y$8)))</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$8:$AA$8))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$8:$AA$8=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$8:$AA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$8:$Y$8))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$8:$Y$8=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$8:$Y$8)))</f>
         <v/>
       </c>
     </row>
@@ -5250,15 +4976,15 @@
         <v>5</v>
       </c>
       <c r="B9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$9:$AA$9))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$9:$AA$9=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$9:$AA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$9:$Y$9))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$9:$Y$9=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$9:$Y$9)))</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$9:$AA$9))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$9:$AA$9=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$9:$AA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$9:$Y$9))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$9:$Y$9=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$9:$Y$9)))</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$9:$AA$9))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$9:$AA$9=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$9:$AA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$9:$Y$9))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$9:$Y$9=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$9:$Y$9)))</f>
         <v/>
       </c>
     </row>
@@ -5267,15 +4993,15 @@
         <v>6</v>
       </c>
       <c r="B10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$10:$AA$10))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$10:$AA$10=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$10:$AA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$10:$Y$10))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$10:$Y$10=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$10:$Y$10)))</f>
         <v/>
       </c>
       <c r="C10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$10:$AA$10))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$10:$AA$10=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$10:$AA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$10:$Y$10))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$10:$Y$10=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$10:$Y$10)))</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$10:$AA$10))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$10:$AA$10=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$10:$AA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$10:$Y$10))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$10:$Y$10=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$10:$Y$10)))</f>
         <v/>
       </c>
     </row>
@@ -5284,15 +5010,15 @@
         <v>7</v>
       </c>
       <c r="B11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$11:$AA$11))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$11:$AA$11=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$11:$AA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$11:$Y$11))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$11:$Y$11=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$11:$Y$11)))</f>
         <v/>
       </c>
       <c r="C11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$11:$AA$11))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$11:$AA$11=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$11:$AA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$11:$Y$11))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$11:$Y$11=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$11:$Y$11)))</f>
         <v/>
       </c>
       <c r="D11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$11:$AA$11))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$11:$AA$11=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$11:$AA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$11:$Y$11))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$11:$Y$11=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$11:$Y$11)))</f>
         <v/>
       </c>
     </row>
@@ -5301,15 +5027,15 @@
         <v>8</v>
       </c>
       <c r="B12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$12:$AA$12))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$12:$AA$12=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$12:$AA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$12:$Y$12))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$12:$Y$12=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$12:$Y$12)))</f>
         <v/>
       </c>
       <c r="C12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$12:$AA$12))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$12:$AA$12=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$12:$AA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$12:$Y$12))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$12:$Y$12=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$12:$Y$12)))</f>
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$12:$AA$12))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$12:$AA$12=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$12:$AA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$12:$Y$12))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$12:$Y$12=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$12:$Y$12)))</f>
         <v/>
       </c>
     </row>
@@ -5318,15 +5044,15 @@
         <v>9</v>
       </c>
       <c r="B13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$13:$AA$13))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$13:$AA$13=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$13:$AA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$13:$Y$13))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$13:$Y$13=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$13:$Y$13)))</f>
         <v/>
       </c>
       <c r="C13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$13:$AA$13))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$13:$AA$13=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$13:$AA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$13:$Y$13))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$13:$Y$13=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$13:$Y$13)))</f>
         <v/>
       </c>
       <c r="D13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$13:$AA$13))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$13:$AA$13=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$13:$AA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$13:$Y$13))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$13:$Y$13=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$13:$Y$13)))</f>
         <v/>
       </c>
     </row>
@@ -5335,15 +5061,15 @@
         <v>10</v>
       </c>
       <c r="B14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$14:$AA$14))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$14:$AA$14=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$14:$AA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$14:$Y$14))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$14:$Y$14=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$14:$Y$14)))</f>
         <v/>
       </c>
       <c r="C14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$14:$AA$14))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$14:$AA$14=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$14:$AA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$14:$Y$14))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$14:$Y$14=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$14:$Y$14)))</f>
         <v/>
       </c>
       <c r="D14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$14:$AA$14))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$14:$AA$14=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$14:$AA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$14:$Y$14))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$14:$Y$14=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$14:$Y$14)))</f>
         <v/>
       </c>
     </row>
@@ -5352,15 +5078,15 @@
         <v>11</v>
       </c>
       <c r="B15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$15:$AA$15))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$15:$AA$15=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$15:$AA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$15:$Y$15))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$15:$Y$15=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$15:$Y$15)))</f>
         <v/>
       </c>
       <c r="C15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$15:$AA$15))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$15:$AA$15=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$15:$AA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$15:$Y$15))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$15:$Y$15=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$15:$Y$15)))</f>
         <v/>
       </c>
       <c r="D15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$15:$AA$15))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$15:$AA$15=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$15:$AA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$15:$Y$15))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$15:$Y$15=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$15:$Y$15)))</f>
         <v/>
       </c>
     </row>
@@ -5369,15 +5095,15 @@
         <v>12</v>
       </c>
       <c r="B16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$16:$AA$16))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$16:$AA$16=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$16:$AA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$16:$Y$16))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$16:$Y$16=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$16:$Y$16)))</f>
         <v/>
       </c>
       <c r="C16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$16:$AA$16))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$16:$AA$16=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$16:$AA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$16:$Y$16))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$16:$Y$16=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$16:$Y$16)))</f>
         <v/>
       </c>
       <c r="D16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$16:$AA$16))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$16:$AA$16=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$16:$AA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$16:$Y$16))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$16:$Y$16=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$16:$Y$16)))</f>
         <v/>
       </c>
     </row>
@@ -5386,15 +5112,15 @@
         <v>13</v>
       </c>
       <c r="B17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$17:$AA$17))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$17:$AA$17=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$17:$AA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$17:$Y$17))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$17:$Y$17=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$17:$Y$17)))</f>
         <v/>
       </c>
       <c r="C17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$17:$AA$17))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$17:$AA$17=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$17:$AA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$17:$Y$17))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$17:$Y$17=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$17:$Y$17)))</f>
         <v/>
       </c>
       <c r="D17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$17:$AA$17))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$17:$AA$17=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$17:$AA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$17:$Y$17))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$17:$Y$17=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$17:$Y$17)))</f>
         <v/>
       </c>
     </row>
@@ -5403,15 +5129,15 @@
         <v>14</v>
       </c>
       <c r="B18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$18:$AA$18))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$18:$AA$18=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$18:$AA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$18:$Y$18))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$18:$Y$18=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$18:$Y$18)))</f>
         <v/>
       </c>
       <c r="C18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$18:$AA$18))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$18:$AA$18=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$18:$AA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$18:$Y$18))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$18:$Y$18=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$18:$Y$18)))</f>
         <v/>
       </c>
       <c r="D18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$18:$AA$18))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$18:$AA$18=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$18:$AA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$18:$Y$18))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$18:$Y$18=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$18:$Y$18)))</f>
         <v/>
       </c>
     </row>
@@ -5420,15 +5146,15 @@
         <v>15</v>
       </c>
       <c r="B19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$19:$AA$19))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$19:$AA$19=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$19:$AA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$19:$Y$19))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$19:$Y$19=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$19:$Y$19)))</f>
         <v/>
       </c>
       <c r="C19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$19:$AA$19))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$19:$AA$19=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$19:$AA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$19:$Y$19))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$19:$Y$19=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$19:$Y$19)))</f>
         <v/>
       </c>
       <c r="D19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$19:$AA$19))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$19:$AA$19=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$19:$AA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$19:$Y$19))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$19:$Y$19=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$19:$Y$19)))</f>
         <v/>
       </c>
     </row>
@@ -5437,15 +5163,15 @@
         <v>16</v>
       </c>
       <c r="B20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$20:$AA$20))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$20:$AA$20=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$20:$AA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$20:$Y$20))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$20:$Y$20=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$20:$Y$20)))</f>
         <v/>
       </c>
       <c r="C20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$20:$AA$20))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$20:$AA$20=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$20:$AA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$20:$Y$20))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$20:$Y$20=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$20:$Y$20)))</f>
         <v/>
       </c>
       <c r="D20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$20:$AA$20))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$20:$AA$20=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$20:$AA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$20:$Y$20))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$20:$Y$20=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$20:$Y$20)))</f>
         <v/>
       </c>
     </row>
@@ -5454,15 +5180,15 @@
         <v>17</v>
       </c>
       <c r="B21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$21:$AA$21))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$21:$AA$21=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$21:$AA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$21:$Y$21))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$21:$Y$21=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$21:$Y$21)))</f>
         <v/>
       </c>
       <c r="C21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$21:$AA$21))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$21:$AA$21=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$21:$AA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$21:$Y$21))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$21:$Y$21=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$21:$Y$21)))</f>
         <v/>
       </c>
       <c r="D21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$21:$AA$21))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$21:$AA$21=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$21:$AA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$21:$Y$21))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$21:$Y$21=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$21:$Y$21)))</f>
         <v/>
       </c>
     </row>
@@ -5471,15 +5197,15 @@
         <v>18</v>
       </c>
       <c r="B22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$22:$AA$22))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$22:$AA$22=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$22:$AA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$22:$Y$22))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$22:$Y$22=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$22:$Y$22)))</f>
         <v/>
       </c>
       <c r="C22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$22:$AA$22))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$22:$AA$22=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$22:$AA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$22:$Y$22))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$22:$Y$22=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$22:$Y$22)))</f>
         <v/>
       </c>
       <c r="D22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$22:$AA$22))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$22:$AA$22=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$22:$AA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$22:$Y$22))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$22:$Y$22=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$22:$Y$22)))</f>
         <v/>
       </c>
     </row>
@@ -5488,15 +5214,15 @@
         <v>19</v>
       </c>
       <c r="B23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$23:$AA$23))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$23:$AA$23=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$23:$AA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$23:$Y$23))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$23:$Y$23=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$23:$Y$23)))</f>
         <v/>
       </c>
       <c r="C23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$23:$AA$23))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$23:$AA$23=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$23:$AA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$23:$Y$23))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$23:$Y$23=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$23:$Y$23)))</f>
         <v/>
       </c>
       <c r="D23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$23:$AA$23))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$23:$AA$23=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$23:$AA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$23:$Y$23))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$23:$Y$23=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$23:$Y$23)))</f>
         <v/>
       </c>
     </row>
@@ -5505,15 +5231,15 @@
         <v>20</v>
       </c>
       <c r="B24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$24:$AA$24))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$24:$AA$24=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$24:$AA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$24:$Y$24))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$24:$Y$24=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$24:$Y$24)))</f>
         <v/>
       </c>
       <c r="C24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$24:$AA$24))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$24:$AA$24=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$24:$AA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$24:$Y$24))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$24:$Y$24=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$24:$Y$24)))</f>
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$24:$AA$24))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$24:$AA$24=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$24:$AA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$24:$Y$24))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$24:$Y$24=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$24:$Y$24)))</f>
         <v/>
       </c>
     </row>
@@ -5522,15 +5248,15 @@
         <v>21</v>
       </c>
       <c r="B25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$25:$AA$25))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$25:$AA$25=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$25:$AA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$25:$Y$25))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$25:$Y$25=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$25:$Y$25)))</f>
         <v/>
       </c>
       <c r="C25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$25:$AA$25))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$25:$AA$25=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$25:$AA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$25:$Y$25))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$25:$Y$25=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$25:$Y$25)))</f>
         <v/>
       </c>
       <c r="D25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$25:$AA$25))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$25:$AA$25=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$25:$AA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$25:$Y$25))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$25:$Y$25=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$25:$Y$25)))</f>
         <v/>
       </c>
     </row>
@@ -5539,15 +5265,15 @@
         <v>22</v>
       </c>
       <c r="B26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$26:$AA$26))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$26:$AA$26=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$26:$AA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$26:$Y$26))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$26:$Y$26=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$26:$Y$26)))</f>
         <v/>
       </c>
       <c r="C26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$26:$AA$26))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$26:$AA$26=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$26:$AA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$26:$Y$26))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$26:$Y$26=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$26:$Y$26)))</f>
         <v/>
       </c>
       <c r="D26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$26:$AA$26))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$26:$AA$26=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$26:$AA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$26:$Y$26))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$26:$Y$26=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$26:$Y$26)))</f>
         <v/>
       </c>
     </row>
@@ -5556,15 +5282,15 @@
         <v>23</v>
       </c>
       <c r="B27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$27:$AA$27))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$27:$AA$27=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$27:$AA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$27:$Y$27))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$27:$Y$27=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$27:$Y$27)))</f>
         <v/>
       </c>
       <c r="C27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$27:$AA$27))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$27:$AA$27=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$27:$AA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$27:$Y$27))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$27:$Y$27=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$27:$Y$27)))</f>
         <v/>
       </c>
       <c r="D27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$27:$AA$27))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$27:$AA$27=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$27:$AA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$27:$Y$27))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$27:$Y$27=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$27:$Y$27)))</f>
         <v/>
       </c>
     </row>
@@ -5573,15 +5299,15 @@
         <v>24</v>
       </c>
       <c r="B28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$28:$AA$28))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$28:$AA$28=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$28:$AA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$28:$Y$28))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$28:$Y$28=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$28:$Y$28)))</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$28:$AA$28))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$28:$AA$28=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$28:$AA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$28:$Y$28))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$28:$Y$28=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$28:$Y$28)))</f>
         <v/>
       </c>
       <c r="D28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$28:$AA$28))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$28:$AA$28=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$28:$AA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$28:$Y$28))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$28:$Y$28=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$28:$Y$28)))</f>
         <v/>
       </c>
     </row>
@@ -5590,15 +5316,15 @@
         <v>25</v>
       </c>
       <c r="B29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$29:$AA$29))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$29:$AA$29=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$29:$AA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$29:$Y$29))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$29:$Y$29=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$29:$Y$29)))</f>
         <v/>
       </c>
       <c r="C29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$29:$AA$29))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$29:$AA$29=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$29:$AA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$29:$Y$29))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$29:$Y$29=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$29:$Y$29)))</f>
         <v/>
       </c>
       <c r="D29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$29:$AA$29))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$29:$AA$29=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$29:$AA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$29:$Y$29))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$29:$Y$29=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$29:$Y$29)))</f>
         <v/>
       </c>
     </row>
@@ -5607,15 +5333,15 @@
         <v>26</v>
       </c>
       <c r="B30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$30:$AA$30))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$30:$AA$30=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$30:$AA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$30:$Y$30))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$30:$Y$30=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$30:$Y$30)))</f>
         <v/>
       </c>
       <c r="C30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$30:$AA$30))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$30:$AA$30=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$30:$AA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$30:$Y$30))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$30:$Y$30=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$30:$Y$30)))</f>
         <v/>
       </c>
       <c r="D30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$30:$AA$30))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$30:$AA$30=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$30:$AA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$30:$Y$30))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$30:$Y$30=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$30:$Y$30)))</f>
         <v/>
       </c>
     </row>
@@ -5624,15 +5350,15 @@
         <v>27</v>
       </c>
       <c r="B31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$31:$AA$31))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$31:$AA$31=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$31:$AA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$31:$Y$31))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$31:$Y$31=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$31:$Y$31)))</f>
         <v/>
       </c>
       <c r="C31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$31:$AA$31))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$31:$AA$31=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$31:$AA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$31:$Y$31))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$31:$Y$31=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$31:$Y$31)))</f>
         <v/>
       </c>
       <c r="D31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$31:$AA$31))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$31:$AA$31=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$31:$AA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$31:$Y$31))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$31:$Y$31=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$31:$Y$31)))</f>
         <v/>
       </c>
     </row>
@@ -5641,15 +5367,15 @@
         <v>28</v>
       </c>
       <c r="B32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$32:$AA$32))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$32:$AA$32=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$32:$AA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$32:$Y$32))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$32:$Y$32=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$32:$Y$32)))</f>
         <v/>
       </c>
       <c r="C32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$32:$AA$32))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$32:$AA$32=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$32:$AA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$32:$Y$32))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$32:$Y$32=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$32:$Y$32)))</f>
         <v/>
       </c>
       <c r="D32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$32:$AA$32))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$32:$AA$32=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$32:$AA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$32:$Y$32))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$32:$Y$32=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$32:$Y$32)))</f>
         <v/>
       </c>
     </row>
@@ -5658,15 +5384,15 @@
         <v>29</v>
       </c>
       <c r="B33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$33:$AA$33))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$33:$AA$33=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$33:$AA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$33:$Y$33))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$33:$Y$33=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$33:$Y$33)))</f>
         <v/>
       </c>
       <c r="C33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$33:$AA$33))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$33:$AA$33=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$33:$AA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$33:$Y$33))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$33:$Y$33=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$33:$Y$33)))</f>
         <v/>
       </c>
       <c r="D33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$33:$AA$33))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$33:$AA$33=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$33:$AA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$33:$Y$33))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$33:$Y$33=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$33:$Y$33)))</f>
         <v/>
       </c>
     </row>
@@ -5675,15 +5401,15 @@
         <v>30</v>
       </c>
       <c r="B34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$34:$AA$34))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$34:$AA$34=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$34:$AA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$34:$Y$34))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$34:$Y$34=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$34:$Y$34)))</f>
         <v/>
       </c>
       <c r="C34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$34:$AA$34))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$34:$AA$34=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$34:$AA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$34:$Y$34))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$34:$Y$34=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$34:$Y$34)))</f>
         <v/>
       </c>
       <c r="D34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$34:$AA$34))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$34:$AA$34=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$34:$AA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$34:$Y$34))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$34:$Y$34=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$34:$Y$34)))</f>
         <v/>
       </c>
     </row>
@@ -5692,15 +5418,15 @@
         <v>31</v>
       </c>
       <c r="B35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$35:$AA$35))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$35:$AA$35=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$35:$AA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$35:$Y$35))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$35:$Y$35=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$35:$Y$35)))</f>
         <v/>
       </c>
       <c r="C35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$35:$AA$35))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$35:$AA$35=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$35:$AA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$35:$Y$35))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$35:$Y$35=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$35:$Y$35)))</f>
         <v/>
       </c>
       <c r="D35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$35:$AA$35))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$35:$AA$35=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$35:$AA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$35:$Y$35))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$35:$Y$35=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$35:$Y$35)))</f>
         <v/>
       </c>
     </row>
@@ -5709,15 +5435,15 @@
         <v>32</v>
       </c>
       <c r="B36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$36:$AA$36))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$36:$AA$36=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$36:$AA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$36:$Y$36))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$36:$Y$36=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$36:$Y$36)))</f>
         <v/>
       </c>
       <c r="C36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$36:$AA$36))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$36:$AA$36=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$36:$AA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$36:$Y$36))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$36:$Y$36=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$36:$Y$36)))</f>
         <v/>
       </c>
       <c r="D36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$36:$AA$36))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$36:$AA$36=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$36:$AA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$36:$Y$36))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$36:$Y$36=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$36:$Y$36)))</f>
         <v/>
       </c>
     </row>
@@ -5726,15 +5452,15 @@
         <v>33</v>
       </c>
       <c r="B37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$37:$AA$37))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$37:$AA$37=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$37:$AA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$37:$Y$37))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$37:$Y$37=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$37:$Y$37)))</f>
         <v/>
       </c>
       <c r="C37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$37:$AA$37))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$37:$AA$37=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$37:$AA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$37:$Y$37))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$37:$Y$37=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$37:$Y$37)))</f>
         <v/>
       </c>
       <c r="D37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$37:$AA$37))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$37:$AA$37=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$37:$AA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$37:$Y$37))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$37:$Y$37=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$37:$Y$37)))</f>
         <v/>
       </c>
     </row>
@@ -5743,15 +5469,15 @@
         <v>34</v>
       </c>
       <c r="B38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$38:$AA$38))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$38:$AA$38=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$38:$AA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$38:$Y$38))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$38:$Y$38=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$38:$Y$38)))</f>
         <v/>
       </c>
       <c r="C38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$38:$AA$38))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$38:$AA$38=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$38:$AA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$38:$Y$38))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$38:$Y$38=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$38:$Y$38)))</f>
         <v/>
       </c>
       <c r="D38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$38:$AA$38))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$38:$AA$38=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$38:$AA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$38:$Y$38))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$38:$Y$38=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$38:$Y$38)))</f>
         <v/>
       </c>
     </row>
@@ -5760,15 +5486,15 @@
         <v>35</v>
       </c>
       <c r="B39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$39:$AA$39))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$39:$AA$39=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$39:$AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$39:$Y$39))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$39:$Y$39=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$39:$Y$39)))</f>
         <v/>
       </c>
       <c r="C39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$39:$AA$39))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$39:$AA$39=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$39:$AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$39:$Y$39))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$39:$Y$39=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$39:$Y$39)))</f>
         <v/>
       </c>
       <c r="D39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$39:$AA$39))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$39:$AA$39=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$39:$AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$39:$Y$39))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$39:$Y$39=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$39:$Y$39)))</f>
         <v/>
       </c>
     </row>
@@ -5777,15 +5503,15 @@
         <v>36</v>
       </c>
       <c r="B40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$40:$AA$40))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$40:$AA$40=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$40:$AA$40)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$40:$Y$40))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$40:$Y$40=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$40:$Y$40)))</f>
         <v/>
       </c>
       <c r="C40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$40:$AA$40))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$40:$AA$40=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$40:$AA$40)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$40:$Y$40))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$40:$Y$40=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$40:$Y$40)))</f>
         <v/>
       </c>
       <c r="D40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$40:$AA$40))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$40:$AA$40=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$40:$AA$40)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$40:$Y$40))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$40:$Y$40=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$40:$Y$40)))</f>
         <v/>
       </c>
     </row>
@@ -5794,15 +5520,15 @@
         <v>37</v>
       </c>
       <c r="B41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$41:$AA$41))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$41:$AA$41=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$41:$AA$41)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$41:$Y$41))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$41:$Y$41=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$41:$Y$41)))</f>
         <v/>
       </c>
       <c r="C41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$41:$AA$41))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$41:$AA$41=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$41:$AA$41)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$41:$Y$41))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$41:$Y$41=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$41:$Y$41)))</f>
         <v/>
       </c>
       <c r="D41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$41:$AA$41))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$41:$AA$41=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$41:$AA$41)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$41:$Y$41))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$41:$Y$41=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$41:$Y$41)))</f>
         <v/>
       </c>
     </row>
@@ -5811,15 +5537,15 @@
         <v>38</v>
       </c>
       <c r="B42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$42:$AA$42))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$42:$AA$42=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$42:$AA$42)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$42:$Y$42))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$42:$Y$42=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$42:$Y$42)))</f>
         <v/>
       </c>
       <c r="C42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$42:$AA$42))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$42:$AA$42=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$42:$AA$42)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$42:$Y$42))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$42:$Y$42=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$42:$Y$42)))</f>
         <v/>
       </c>
       <c r="D42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$42:$AA$42))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$42:$AA$42=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$42:$AA$42)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$42:$Y$42))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$42:$Y$42=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$42:$Y$42)))</f>
         <v/>
       </c>
     </row>
@@ -5828,15 +5554,15 @@
         <v>39</v>
       </c>
       <c r="B43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$43:$AA$43))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*(Marks!$B$43:$AA$43=1))/SUMPRODUCT((Marks!$B$3:$AA$3=B$4)*ISNUMBER(Marks!$B$43:$AA$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$43:$Y$43))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*(Marks!$B$43:$Y$43=1))/SUMPRODUCT((Marks!$B$3:$Y$3=B$4)*ISNUMBER(Marks!$B$43:$Y$43)))</f>
         <v/>
       </c>
       <c r="C43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$43:$AA$43))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*(Marks!$B$43:$AA$43=1))/SUMPRODUCT((Marks!$B$3:$AA$3=C$4)*ISNUMBER(Marks!$B$43:$AA$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$43:$Y$43))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*(Marks!$B$43:$Y$43=1))/SUMPRODUCT((Marks!$B$3:$Y$3=C$4)*ISNUMBER(Marks!$B$43:$Y$43)))</f>
         <v/>
       </c>
       <c r="D43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$43:$AA$43))=0,"",SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*(Marks!$B$43:$AA$43=1))/SUMPRODUCT((Marks!$B$3:$AA$3=D$4)*ISNUMBER(Marks!$B$43:$AA$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$43:$Y$43))=0,"",SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*(Marks!$B$43:$Y$43=1))/SUMPRODUCT((Marks!$B$3:$Y$3=D$4)*ISNUMBER(Marks!$B$43:$Y$43)))</f>
         <v/>
       </c>
     </row>
@@ -5970,23 +5696,23 @@
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
       <c r="H5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$5:$AA$5))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$5:$AA$5=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$5:$AA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$5:$Y$5))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$5:$Y$5=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$5:$Y$5)))</f>
         <v/>
       </c>
       <c r="I5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$5:$AA$5))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$5:$AA$5=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$5:$AA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$5:$Y$5))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$5:$Y$5=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$5:$Y$5)))</f>
         <v/>
       </c>
       <c r="J5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$5:$AA$5))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$5:$AA$5=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$5:$AA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$5:$Y$5))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$5:$Y$5=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$5:$Y$5)))</f>
         <v/>
       </c>
       <c r="K5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$5:$AA$5))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$5:$AA$5=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$5:$AA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$5:$Y$5))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$5:$Y$5=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$5:$Y$5)))</f>
         <v/>
       </c>
       <c r="L5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$5:$AA$5))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$5:$AA$5=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$5:$AA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$5:$Y$5))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$5:$Y$5=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$5:$Y$5)))</f>
         <v/>
       </c>
     </row>
@@ -6000,23 +5726,23 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="H6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$6:$AA$6))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$6:$AA$6=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$6:$AA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$6:$Y$6))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$6:$Y$6=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$6:$Y$6)))</f>
         <v/>
       </c>
       <c r="I6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$6:$AA$6))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$6:$AA$6=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$6:$AA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$6:$Y$6))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$6:$Y$6=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$6:$Y$6)))</f>
         <v/>
       </c>
       <c r="J6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$6:$AA$6))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$6:$AA$6=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$6:$AA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$6:$Y$6))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$6:$Y$6=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$6:$Y$6)))</f>
         <v/>
       </c>
       <c r="K6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$6:$AA$6))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$6:$AA$6=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$6:$AA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$6:$Y$6))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$6:$Y$6=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$6:$Y$6)))</f>
         <v/>
       </c>
       <c r="L6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$6:$AA$6))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$6:$AA$6=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$6:$AA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$6:$Y$6))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$6:$Y$6=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$6:$Y$6)))</f>
         <v/>
       </c>
     </row>
@@ -6030,23 +5756,23 @@
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="H7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$7:$AA$7))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$7:$AA$7=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$7:$AA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$7:$Y$7))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$7:$Y$7=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$7:$Y$7)))</f>
         <v/>
       </c>
       <c r="I7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$7:$AA$7))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$7:$AA$7=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$7:$AA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$7:$Y$7))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$7:$Y$7=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$7:$Y$7)))</f>
         <v/>
       </c>
       <c r="J7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$7:$AA$7))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$7:$AA$7=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$7:$AA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$7:$Y$7))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$7:$Y$7=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$7:$Y$7)))</f>
         <v/>
       </c>
       <c r="K7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$7:$AA$7))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$7:$AA$7=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$7:$AA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$7:$Y$7))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$7:$Y$7=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$7:$Y$7)))</f>
         <v/>
       </c>
       <c r="L7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$7:$AA$7))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$7:$AA$7=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$7:$AA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$7:$Y$7))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$7:$Y$7=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$7:$Y$7)))</f>
         <v/>
       </c>
     </row>
@@ -6060,23 +5786,23 @@
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
       <c r="H8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$8:$AA$8))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$8:$AA$8=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$8:$AA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$8:$Y$8))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$8:$Y$8=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$8:$Y$8)))</f>
         <v/>
       </c>
       <c r="I8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$8:$AA$8))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$8:$AA$8=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$8:$AA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$8:$Y$8))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$8:$Y$8=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$8:$Y$8)))</f>
         <v/>
       </c>
       <c r="J8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$8:$AA$8))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$8:$AA$8=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$8:$AA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$8:$Y$8))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$8:$Y$8=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$8:$Y$8)))</f>
         <v/>
       </c>
       <c r="K8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$8:$AA$8))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$8:$AA$8=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$8:$AA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$8:$Y$8))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$8:$Y$8=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$8:$Y$8)))</f>
         <v/>
       </c>
       <c r="L8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$8:$AA$8))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$8:$AA$8=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$8:$AA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$8:$Y$8))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$8:$Y$8=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$8:$Y$8)))</f>
         <v/>
       </c>
     </row>
@@ -6090,23 +5816,23 @@
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
       <c r="H9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$9:$AA$9))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$9:$AA$9=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$9:$AA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$9:$Y$9))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$9:$Y$9=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$9:$Y$9)))</f>
         <v/>
       </c>
       <c r="I9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$9:$AA$9))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$9:$AA$9=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$9:$AA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$9:$Y$9))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$9:$Y$9=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$9:$Y$9)))</f>
         <v/>
       </c>
       <c r="J9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$9:$AA$9))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$9:$AA$9=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$9:$AA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$9:$Y$9))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$9:$Y$9=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$9:$Y$9)))</f>
         <v/>
       </c>
       <c r="K9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$9:$AA$9))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$9:$AA$9=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$9:$AA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$9:$Y$9))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$9:$Y$9=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$9:$Y$9)))</f>
         <v/>
       </c>
       <c r="L9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$9:$AA$9))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$9:$AA$9=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$9:$AA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$9:$Y$9))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$9:$Y$9=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$9:$Y$9)))</f>
         <v/>
       </c>
     </row>
@@ -6120,23 +5846,23 @@
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
       <c r="H10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$10:$AA$10))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$10:$AA$10=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$10:$AA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$10:$Y$10))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$10:$Y$10=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$10:$Y$10)))</f>
         <v/>
       </c>
       <c r="I10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$10:$AA$10))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$10:$AA$10=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$10:$AA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$10:$Y$10))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$10:$Y$10=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$10:$Y$10)))</f>
         <v/>
       </c>
       <c r="J10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$10:$AA$10))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$10:$AA$10=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$10:$AA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$10:$Y$10))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$10:$Y$10=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$10:$Y$10)))</f>
         <v/>
       </c>
       <c r="K10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$10:$AA$10))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$10:$AA$10=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$10:$AA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$10:$Y$10))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$10:$Y$10=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$10:$Y$10)))</f>
         <v/>
       </c>
       <c r="L10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$10:$AA$10))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$10:$AA$10=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$10:$AA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$10:$Y$10))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$10:$Y$10=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$10:$Y$10)))</f>
         <v/>
       </c>
     </row>
@@ -6150,23 +5876,23 @@
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
       <c r="H11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$11:$AA$11))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$11:$AA$11=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$11:$AA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$11:$Y$11))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$11:$Y$11=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$11:$Y$11)))</f>
         <v/>
       </c>
       <c r="I11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$11:$AA$11))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$11:$AA$11=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$11:$AA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$11:$Y$11))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$11:$Y$11=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$11:$Y$11)))</f>
         <v/>
       </c>
       <c r="J11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$11:$AA$11))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$11:$AA$11=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$11:$AA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$11:$Y$11))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$11:$Y$11=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$11:$Y$11)))</f>
         <v/>
       </c>
       <c r="K11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$11:$AA$11))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$11:$AA$11=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$11:$AA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$11:$Y$11))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$11:$Y$11=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$11:$Y$11)))</f>
         <v/>
       </c>
       <c r="L11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$11:$AA$11))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$11:$AA$11=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$11:$AA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$11:$Y$11))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$11:$Y$11=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$11:$Y$11)))</f>
         <v/>
       </c>
     </row>
@@ -6180,23 +5906,23 @@
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
       <c r="H12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$12:$AA$12))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$12:$AA$12=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$12:$AA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$12:$Y$12))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$12:$Y$12=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$12:$Y$12)))</f>
         <v/>
       </c>
       <c r="I12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$12:$AA$12))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$12:$AA$12=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$12:$AA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$12:$Y$12))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$12:$Y$12=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$12:$Y$12)))</f>
         <v/>
       </c>
       <c r="J12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$12:$AA$12))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$12:$AA$12=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$12:$AA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$12:$Y$12))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$12:$Y$12=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$12:$Y$12)))</f>
         <v/>
       </c>
       <c r="K12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$12:$AA$12))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$12:$AA$12=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$12:$AA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$12:$Y$12))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$12:$Y$12=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$12:$Y$12)))</f>
         <v/>
       </c>
       <c r="L12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$12:$AA$12))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$12:$AA$12=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$12:$AA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$12:$Y$12))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$12:$Y$12=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$12:$Y$12)))</f>
         <v/>
       </c>
     </row>
@@ -6210,23 +5936,23 @@
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
       <c r="H13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$13:$AA$13))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$13:$AA$13=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$13:$AA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$13:$Y$13))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$13:$Y$13=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$13:$Y$13)))</f>
         <v/>
       </c>
       <c r="I13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$13:$AA$13))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$13:$AA$13=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$13:$AA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$13:$Y$13))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$13:$Y$13=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$13:$Y$13)))</f>
         <v/>
       </c>
       <c r="J13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$13:$AA$13))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$13:$AA$13=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$13:$AA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$13:$Y$13))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$13:$Y$13=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$13:$Y$13)))</f>
         <v/>
       </c>
       <c r="K13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$13:$AA$13))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$13:$AA$13=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$13:$AA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$13:$Y$13))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$13:$Y$13=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$13:$Y$13)))</f>
         <v/>
       </c>
       <c r="L13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$13:$AA$13))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$13:$AA$13=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$13:$AA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$13:$Y$13))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$13:$Y$13=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$13:$Y$13)))</f>
         <v/>
       </c>
     </row>
@@ -6240,23 +5966,23 @@
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
       <c r="H14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$14:$AA$14))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$14:$AA$14=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$14:$AA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$14:$Y$14))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$14:$Y$14=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$14:$Y$14)))</f>
         <v/>
       </c>
       <c r="I14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$14:$AA$14))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$14:$AA$14=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$14:$AA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$14:$Y$14))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$14:$Y$14=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$14:$Y$14)))</f>
         <v/>
       </c>
       <c r="J14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$14:$AA$14))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$14:$AA$14=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$14:$AA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$14:$Y$14))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$14:$Y$14=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$14:$Y$14)))</f>
         <v/>
       </c>
       <c r="K14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$14:$AA$14))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$14:$AA$14=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$14:$AA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$14:$Y$14))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$14:$Y$14=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$14:$Y$14)))</f>
         <v/>
       </c>
       <c r="L14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$14:$AA$14))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$14:$AA$14=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$14:$AA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$14:$Y$14))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$14:$Y$14=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$14:$Y$14)))</f>
         <v/>
       </c>
     </row>
@@ -6270,23 +5996,23 @@
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
       <c r="H15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$15:$AA$15))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$15:$AA$15=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$15:$AA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$15:$Y$15))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$15:$Y$15=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$15:$Y$15)))</f>
         <v/>
       </c>
       <c r="I15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$15:$AA$15))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$15:$AA$15=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$15:$AA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$15:$Y$15))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$15:$Y$15=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$15:$Y$15)))</f>
         <v/>
       </c>
       <c r="J15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$15:$AA$15))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$15:$AA$15=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$15:$AA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$15:$Y$15))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$15:$Y$15=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$15:$Y$15)))</f>
         <v/>
       </c>
       <c r="K15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$15:$AA$15))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$15:$AA$15=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$15:$AA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$15:$Y$15))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$15:$Y$15=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$15:$Y$15)))</f>
         <v/>
       </c>
       <c r="L15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$15:$AA$15))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$15:$AA$15=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$15:$AA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$15:$Y$15))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$15:$Y$15=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$15:$Y$15)))</f>
         <v/>
       </c>
     </row>
@@ -6300,23 +6026,23 @@
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="H16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$16:$AA$16))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$16:$AA$16=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$16:$AA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$16:$Y$16))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$16:$Y$16=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$16:$Y$16)))</f>
         <v/>
       </c>
       <c r="I16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$16:$AA$16))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$16:$AA$16=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$16:$AA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$16:$Y$16))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$16:$Y$16=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$16:$Y$16)))</f>
         <v/>
       </c>
       <c r="J16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$16:$AA$16))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$16:$AA$16=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$16:$AA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$16:$Y$16))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$16:$Y$16=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$16:$Y$16)))</f>
         <v/>
       </c>
       <c r="K16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$16:$AA$16))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$16:$AA$16=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$16:$AA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$16:$Y$16))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$16:$Y$16=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$16:$Y$16)))</f>
         <v/>
       </c>
       <c r="L16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$16:$AA$16))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$16:$AA$16=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$16:$AA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$16:$Y$16))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$16:$Y$16=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$16:$Y$16)))</f>
         <v/>
       </c>
     </row>
@@ -6330,23 +6056,23 @@
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="H17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$17:$AA$17))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$17:$AA$17=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$17:$AA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$17:$Y$17))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$17:$Y$17=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$17:$Y$17)))</f>
         <v/>
       </c>
       <c r="I17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$17:$AA$17))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$17:$AA$17=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$17:$AA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$17:$Y$17))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$17:$Y$17=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$17:$Y$17)))</f>
         <v/>
       </c>
       <c r="J17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$17:$AA$17))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$17:$AA$17=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$17:$AA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$17:$Y$17))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$17:$Y$17=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$17:$Y$17)))</f>
         <v/>
       </c>
       <c r="K17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$17:$AA$17))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$17:$AA$17=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$17:$AA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$17:$Y$17))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$17:$Y$17=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$17:$Y$17)))</f>
         <v/>
       </c>
       <c r="L17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$17:$AA$17))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$17:$AA$17=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$17:$AA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$17:$Y$17))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$17:$Y$17=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$17:$Y$17)))</f>
         <v/>
       </c>
     </row>
@@ -6360,23 +6086,23 @@
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="H18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$18:$AA$18))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$18:$AA$18=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$18:$AA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$18:$Y$18))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$18:$Y$18=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$18:$Y$18)))</f>
         <v/>
       </c>
       <c r="I18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$18:$AA$18))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$18:$AA$18=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$18:$AA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$18:$Y$18))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$18:$Y$18=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$18:$Y$18)))</f>
         <v/>
       </c>
       <c r="J18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$18:$AA$18))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$18:$AA$18=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$18:$AA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$18:$Y$18))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$18:$Y$18=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$18:$Y$18)))</f>
         <v/>
       </c>
       <c r="K18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$18:$AA$18))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$18:$AA$18=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$18:$AA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$18:$Y$18))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$18:$Y$18=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$18:$Y$18)))</f>
         <v/>
       </c>
       <c r="L18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$18:$AA$18))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$18:$AA$18=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$18:$AA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$18:$Y$18))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$18:$Y$18=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$18:$Y$18)))</f>
         <v/>
       </c>
     </row>
@@ -6390,23 +6116,23 @@
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="H19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$19:$AA$19))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$19:$AA$19=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$19:$AA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$19:$Y$19))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$19:$Y$19=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$19:$Y$19)))</f>
         <v/>
       </c>
       <c r="I19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$19:$AA$19))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$19:$AA$19=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$19:$AA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$19:$Y$19))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$19:$Y$19=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$19:$Y$19)))</f>
         <v/>
       </c>
       <c r="J19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$19:$AA$19))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$19:$AA$19=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$19:$AA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$19:$Y$19))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$19:$Y$19=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$19:$Y$19)))</f>
         <v/>
       </c>
       <c r="K19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$19:$AA$19))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$19:$AA$19=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$19:$AA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$19:$Y$19))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$19:$Y$19=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$19:$Y$19)))</f>
         <v/>
       </c>
       <c r="L19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$19:$AA$19))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$19:$AA$19=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$19:$AA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$19:$Y$19))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$19:$Y$19=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$19:$Y$19)))</f>
         <v/>
       </c>
     </row>
@@ -6420,23 +6146,23 @@
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="H20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$20:$AA$20))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$20:$AA$20=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$20:$AA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$20:$Y$20))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$20:$Y$20=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$20:$Y$20)))</f>
         <v/>
       </c>
       <c r="I20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$20:$AA$20))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$20:$AA$20=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$20:$AA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$20:$Y$20))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$20:$Y$20=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$20:$Y$20)))</f>
         <v/>
       </c>
       <c r="J20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$20:$AA$20))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$20:$AA$20=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$20:$AA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$20:$Y$20))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$20:$Y$20=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$20:$Y$20)))</f>
         <v/>
       </c>
       <c r="K20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$20:$AA$20))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$20:$AA$20=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$20:$AA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$20:$Y$20))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$20:$Y$20=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$20:$Y$20)))</f>
         <v/>
       </c>
       <c r="L20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$20:$AA$20))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$20:$AA$20=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$20:$AA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$20:$Y$20))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$20:$Y$20=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$20:$Y$20)))</f>
         <v/>
       </c>
     </row>
@@ -6450,23 +6176,23 @@
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
       <c r="H21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$21:$AA$21))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$21:$AA$21=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$21:$AA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$21:$Y$21))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$21:$Y$21=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$21:$Y$21)))</f>
         <v/>
       </c>
       <c r="I21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$21:$AA$21))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$21:$AA$21=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$21:$AA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$21:$Y$21))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$21:$Y$21=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$21:$Y$21)))</f>
         <v/>
       </c>
       <c r="J21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$21:$AA$21))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$21:$AA$21=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$21:$AA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$21:$Y$21))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$21:$Y$21=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$21:$Y$21)))</f>
         <v/>
       </c>
       <c r="K21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$21:$AA$21))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$21:$AA$21=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$21:$AA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$21:$Y$21))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$21:$Y$21=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$21:$Y$21)))</f>
         <v/>
       </c>
       <c r="L21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$21:$AA$21))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$21:$AA$21=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$21:$AA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$21:$Y$21))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$21:$Y$21=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$21:$Y$21)))</f>
         <v/>
       </c>
     </row>
@@ -6480,23 +6206,23 @@
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
       <c r="H22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$22:$AA$22))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$22:$AA$22=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$22:$AA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$22:$Y$22))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$22:$Y$22=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$22:$Y$22)))</f>
         <v/>
       </c>
       <c r="I22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$22:$AA$22))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$22:$AA$22=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$22:$AA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$22:$Y$22))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$22:$Y$22=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$22:$Y$22)))</f>
         <v/>
       </c>
       <c r="J22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$22:$AA$22))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$22:$AA$22=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$22:$AA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$22:$Y$22))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$22:$Y$22=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$22:$Y$22)))</f>
         <v/>
       </c>
       <c r="K22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$22:$AA$22))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$22:$AA$22=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$22:$AA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$22:$Y$22))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$22:$Y$22=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$22:$Y$22)))</f>
         <v/>
       </c>
       <c r="L22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$22:$AA$22))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$22:$AA$22=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$22:$AA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$22:$Y$22))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$22:$Y$22=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$22:$Y$22)))</f>
         <v/>
       </c>
     </row>
@@ -6510,23 +6236,23 @@
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
       <c r="H23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$23:$AA$23))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$23:$AA$23=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$23:$AA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$23:$Y$23))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$23:$Y$23=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$23:$Y$23)))</f>
         <v/>
       </c>
       <c r="I23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$23:$AA$23))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$23:$AA$23=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$23:$AA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$23:$Y$23))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$23:$Y$23=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$23:$Y$23)))</f>
         <v/>
       </c>
       <c r="J23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$23:$AA$23))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$23:$AA$23=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$23:$AA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$23:$Y$23))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$23:$Y$23=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$23:$Y$23)))</f>
         <v/>
       </c>
       <c r="K23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$23:$AA$23))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$23:$AA$23=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$23:$AA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$23:$Y$23))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$23:$Y$23=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$23:$Y$23)))</f>
         <v/>
       </c>
       <c r="L23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$23:$AA$23))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$23:$AA$23=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$23:$AA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$23:$Y$23))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$23:$Y$23=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$23:$Y$23)))</f>
         <v/>
       </c>
     </row>
@@ -6540,23 +6266,23 @@
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
       <c r="H24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$24:$AA$24))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$24:$AA$24=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$24:$AA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$24:$Y$24))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$24:$Y$24=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$24:$Y$24)))</f>
         <v/>
       </c>
       <c r="I24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$24:$AA$24))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$24:$AA$24=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$24:$AA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$24:$Y$24))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$24:$Y$24=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$24:$Y$24)))</f>
         <v/>
       </c>
       <c r="J24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$24:$AA$24))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$24:$AA$24=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$24:$AA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$24:$Y$24))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$24:$Y$24=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$24:$Y$24)))</f>
         <v/>
       </c>
       <c r="K24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$24:$AA$24))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$24:$AA$24=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$24:$AA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$24:$Y$24))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$24:$Y$24=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$24:$Y$24)))</f>
         <v/>
       </c>
       <c r="L24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$24:$AA$24))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$24:$AA$24=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$24:$AA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$24:$Y$24))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$24:$Y$24=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$24:$Y$24)))</f>
         <v/>
       </c>
     </row>
@@ -6570,23 +6296,23 @@
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
       <c r="H25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$25:$AA$25))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$25:$AA$25=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$25:$AA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$25:$Y$25))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$25:$Y$25=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$25:$Y$25)))</f>
         <v/>
       </c>
       <c r="I25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$25:$AA$25))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$25:$AA$25=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$25:$AA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$25:$Y$25))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$25:$Y$25=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$25:$Y$25)))</f>
         <v/>
       </c>
       <c r="J25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$25:$AA$25))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$25:$AA$25=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$25:$AA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$25:$Y$25))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$25:$Y$25=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$25:$Y$25)))</f>
         <v/>
       </c>
       <c r="K25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$25:$AA$25))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$25:$AA$25=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$25:$AA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$25:$Y$25))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$25:$Y$25=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$25:$Y$25)))</f>
         <v/>
       </c>
       <c r="L25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$25:$AA$25))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$25:$AA$25=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$25:$AA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$25:$Y$25))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$25:$Y$25=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$25:$Y$25)))</f>
         <v/>
       </c>
     </row>
@@ -6600,23 +6326,23 @@
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
       <c r="H26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$26:$AA$26))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$26:$AA$26=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$26:$AA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$26:$Y$26))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$26:$Y$26=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$26:$Y$26)))</f>
         <v/>
       </c>
       <c r="I26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$26:$AA$26))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$26:$AA$26=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$26:$AA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$26:$Y$26))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$26:$Y$26=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$26:$Y$26)))</f>
         <v/>
       </c>
       <c r="J26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$26:$AA$26))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$26:$AA$26=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$26:$AA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$26:$Y$26))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$26:$Y$26=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$26:$Y$26)))</f>
         <v/>
       </c>
       <c r="K26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$26:$AA$26))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$26:$AA$26=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$26:$AA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$26:$Y$26))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$26:$Y$26=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$26:$Y$26)))</f>
         <v/>
       </c>
       <c r="L26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$26:$AA$26))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$26:$AA$26=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$26:$AA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$26:$Y$26))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$26:$Y$26=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$26:$Y$26)))</f>
         <v/>
       </c>
     </row>
@@ -6630,23 +6356,23 @@
       <c r="E27" s="5" t="n"/>
       <c r="F27" s="5" t="n"/>
       <c r="H27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$27:$AA$27))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$27:$AA$27=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$27:$AA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$27:$Y$27))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$27:$Y$27=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$27:$Y$27)))</f>
         <v/>
       </c>
       <c r="I27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$27:$AA$27))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$27:$AA$27=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$27:$AA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$27:$Y$27))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$27:$Y$27=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$27:$Y$27)))</f>
         <v/>
       </c>
       <c r="J27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$27:$AA$27))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$27:$AA$27=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$27:$AA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$27:$Y$27))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$27:$Y$27=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$27:$Y$27)))</f>
         <v/>
       </c>
       <c r="K27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$27:$AA$27))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$27:$AA$27=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$27:$AA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$27:$Y$27))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$27:$Y$27=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$27:$Y$27)))</f>
         <v/>
       </c>
       <c r="L27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$27:$AA$27))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$27:$AA$27=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$27:$AA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$27:$Y$27))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$27:$Y$27=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$27:$Y$27)))</f>
         <v/>
       </c>
     </row>
@@ -6660,23 +6386,23 @@
       <c r="E28" s="5" t="n"/>
       <c r="F28" s="5" t="n"/>
       <c r="H28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$28:$AA$28))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$28:$AA$28=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$28:$AA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$28:$Y$28))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$28:$Y$28=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$28:$Y$28)))</f>
         <v/>
       </c>
       <c r="I28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$28:$AA$28))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$28:$AA$28=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$28:$AA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$28:$Y$28))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$28:$Y$28=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$28:$Y$28)))</f>
         <v/>
       </c>
       <c r="J28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$28:$AA$28))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$28:$AA$28=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$28:$AA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$28:$Y$28))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$28:$Y$28=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$28:$Y$28)))</f>
         <v/>
       </c>
       <c r="K28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$28:$AA$28))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$28:$AA$28=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$28:$AA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$28:$Y$28))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$28:$Y$28=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$28:$Y$28)))</f>
         <v/>
       </c>
       <c r="L28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$28:$AA$28))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$28:$AA$28=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$28:$AA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$28:$Y$28))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$28:$Y$28=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$28:$Y$28)))</f>
         <v/>
       </c>
     </row>
@@ -6690,23 +6416,23 @@
       <c r="E29" s="5" t="n"/>
       <c r="F29" s="5" t="n"/>
       <c r="H29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$29:$AA$29))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$29:$AA$29=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$29:$AA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$29:$Y$29))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$29:$Y$29=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$29:$Y$29)))</f>
         <v/>
       </c>
       <c r="I29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$29:$AA$29))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$29:$AA$29=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$29:$AA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$29:$Y$29))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$29:$Y$29=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$29:$Y$29)))</f>
         <v/>
       </c>
       <c r="J29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$29:$AA$29))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$29:$AA$29=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$29:$AA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$29:$Y$29))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$29:$Y$29=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$29:$Y$29)))</f>
         <v/>
       </c>
       <c r="K29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$29:$AA$29))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$29:$AA$29=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$29:$AA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$29:$Y$29))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$29:$Y$29=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$29:$Y$29)))</f>
         <v/>
       </c>
       <c r="L29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$29:$AA$29))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$29:$AA$29=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$29:$AA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$29:$Y$29))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$29:$Y$29=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$29:$Y$29)))</f>
         <v/>
       </c>
     </row>
@@ -6720,23 +6446,23 @@
       <c r="E30" s="5" t="n"/>
       <c r="F30" s="5" t="n"/>
       <c r="H30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$30:$AA$30))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$30:$AA$30=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$30:$AA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$30:$Y$30))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$30:$Y$30=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$30:$Y$30)))</f>
         <v/>
       </c>
       <c r="I30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$30:$AA$30))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$30:$AA$30=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$30:$AA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$30:$Y$30))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$30:$Y$30=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$30:$Y$30)))</f>
         <v/>
       </c>
       <c r="J30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$30:$AA$30))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$30:$AA$30=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$30:$AA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$30:$Y$30))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$30:$Y$30=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$30:$Y$30)))</f>
         <v/>
       </c>
       <c r="K30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$30:$AA$30))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$30:$AA$30=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$30:$AA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$30:$Y$30))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$30:$Y$30=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$30:$Y$30)))</f>
         <v/>
       </c>
       <c r="L30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$30:$AA$30))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$30:$AA$30=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$30:$AA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$30:$Y$30))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$30:$Y$30=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$30:$Y$30)))</f>
         <v/>
       </c>
     </row>
@@ -6750,23 +6476,23 @@
       <c r="E31" s="5" t="n"/>
       <c r="F31" s="5" t="n"/>
       <c r="H31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$31:$AA$31))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$31:$AA$31=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$31:$AA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$31:$Y$31))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$31:$Y$31=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$31:$Y$31)))</f>
         <v/>
       </c>
       <c r="I31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$31:$AA$31))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$31:$AA$31=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$31:$AA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$31:$Y$31))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$31:$Y$31=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$31:$Y$31)))</f>
         <v/>
       </c>
       <c r="J31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$31:$AA$31))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$31:$AA$31=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$31:$AA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$31:$Y$31))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$31:$Y$31=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$31:$Y$31)))</f>
         <v/>
       </c>
       <c r="K31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$31:$AA$31))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$31:$AA$31=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$31:$AA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$31:$Y$31))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$31:$Y$31=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$31:$Y$31)))</f>
         <v/>
       </c>
       <c r="L31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$31:$AA$31))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$31:$AA$31=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$31:$AA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$31:$Y$31))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$31:$Y$31=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$31:$Y$31)))</f>
         <v/>
       </c>
     </row>
@@ -6780,23 +6506,23 @@
       <c r="E32" s="5" t="n"/>
       <c r="F32" s="5" t="n"/>
       <c r="H32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$32:$AA$32))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$32:$AA$32=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$32:$AA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$32:$Y$32))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$32:$Y$32=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$32:$Y$32)))</f>
         <v/>
       </c>
       <c r="I32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$32:$AA$32))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$32:$AA$32=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$32:$AA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$32:$Y$32))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$32:$Y$32=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$32:$Y$32)))</f>
         <v/>
       </c>
       <c r="J32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$32:$AA$32))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$32:$AA$32=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$32:$AA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$32:$Y$32))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$32:$Y$32=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$32:$Y$32)))</f>
         <v/>
       </c>
       <c r="K32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$32:$AA$32))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$32:$AA$32=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$32:$AA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$32:$Y$32))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$32:$Y$32=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$32:$Y$32)))</f>
         <v/>
       </c>
       <c r="L32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$32:$AA$32))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$32:$AA$32=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$32:$AA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$32:$Y$32))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$32:$Y$32=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$32:$Y$32)))</f>
         <v/>
       </c>
     </row>
@@ -6810,23 +6536,23 @@
       <c r="E33" s="5" t="n"/>
       <c r="F33" s="5" t="n"/>
       <c r="H33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$33:$AA$33))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$33:$AA$33=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$33:$AA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$33:$Y$33))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$33:$Y$33=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$33:$Y$33)))</f>
         <v/>
       </c>
       <c r="I33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$33:$AA$33))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$33:$AA$33=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$33:$AA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$33:$Y$33))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$33:$Y$33=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$33:$Y$33)))</f>
         <v/>
       </c>
       <c r="J33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$33:$AA$33))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$33:$AA$33=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$33:$AA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$33:$Y$33))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$33:$Y$33=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$33:$Y$33)))</f>
         <v/>
       </c>
       <c r="K33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$33:$AA$33))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$33:$AA$33=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$33:$AA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$33:$Y$33))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$33:$Y$33=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$33:$Y$33)))</f>
         <v/>
       </c>
       <c r="L33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$33:$AA$33))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$33:$AA$33=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$33:$AA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$33:$Y$33))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$33:$Y$33=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$33:$Y$33)))</f>
         <v/>
       </c>
     </row>
@@ -6840,23 +6566,23 @@
       <c r="E34" s="5" t="n"/>
       <c r="F34" s="5" t="n"/>
       <c r="H34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$34:$AA$34))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$34:$AA$34=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$34:$AA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$34:$Y$34))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$34:$Y$34=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$34:$Y$34)))</f>
         <v/>
       </c>
       <c r="I34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$34:$AA$34))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$34:$AA$34=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$34:$AA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$34:$Y$34))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$34:$Y$34=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$34:$Y$34)))</f>
         <v/>
       </c>
       <c r="J34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$34:$AA$34))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$34:$AA$34=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$34:$AA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$34:$Y$34))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$34:$Y$34=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$34:$Y$34)))</f>
         <v/>
       </c>
       <c r="K34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$34:$AA$34))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$34:$AA$34=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$34:$AA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$34:$Y$34))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$34:$Y$34=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$34:$Y$34)))</f>
         <v/>
       </c>
       <c r="L34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$34:$AA$34))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$34:$AA$34=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$34:$AA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$34:$Y$34))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$34:$Y$34=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$34:$Y$34)))</f>
         <v/>
       </c>
     </row>
@@ -6870,23 +6596,23 @@
       <c r="E35" s="5" t="n"/>
       <c r="F35" s="5" t="n"/>
       <c r="H35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$35:$AA$35))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$35:$AA$35=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$35:$AA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$35:$Y$35))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$35:$Y$35=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$35:$Y$35)))</f>
         <v/>
       </c>
       <c r="I35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$35:$AA$35))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$35:$AA$35=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$35:$AA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$35:$Y$35))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$35:$Y$35=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$35:$Y$35)))</f>
         <v/>
       </c>
       <c r="J35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$35:$AA$35))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$35:$AA$35=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$35:$AA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$35:$Y$35))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$35:$Y$35=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$35:$Y$35)))</f>
         <v/>
       </c>
       <c r="K35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$35:$AA$35))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$35:$AA$35=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$35:$AA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$35:$Y$35))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$35:$Y$35=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$35:$Y$35)))</f>
         <v/>
       </c>
       <c r="L35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$35:$AA$35))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$35:$AA$35=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$35:$AA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$35:$Y$35))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$35:$Y$35=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$35:$Y$35)))</f>
         <v/>
       </c>
     </row>
@@ -6900,23 +6626,23 @@
       <c r="E36" s="5" t="n"/>
       <c r="F36" s="5" t="n"/>
       <c r="H36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$36:$AA$36))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$36:$AA$36=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$36:$AA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$36:$Y$36))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$36:$Y$36=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$36:$Y$36)))</f>
         <v/>
       </c>
       <c r="I36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$36:$AA$36))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$36:$AA$36=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$36:$AA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$36:$Y$36))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$36:$Y$36=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$36:$Y$36)))</f>
         <v/>
       </c>
       <c r="J36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$36:$AA$36))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$36:$AA$36=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$36:$AA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$36:$Y$36))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$36:$Y$36=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$36:$Y$36)))</f>
         <v/>
       </c>
       <c r="K36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$36:$AA$36))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$36:$AA$36=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$36:$AA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$36:$Y$36))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$36:$Y$36=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$36:$Y$36)))</f>
         <v/>
       </c>
       <c r="L36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$36:$AA$36))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$36:$AA$36=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$36:$AA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$36:$Y$36))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$36:$Y$36=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$36:$Y$36)))</f>
         <v/>
       </c>
     </row>
@@ -6930,23 +6656,23 @@
       <c r="E37" s="5" t="n"/>
       <c r="F37" s="5" t="n"/>
       <c r="H37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$37:$AA$37))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$37:$AA$37=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$37:$AA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$37:$Y$37))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$37:$Y$37=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$37:$Y$37)))</f>
         <v/>
       </c>
       <c r="I37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$37:$AA$37))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$37:$AA$37=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$37:$AA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$37:$Y$37))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$37:$Y$37=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$37:$Y$37)))</f>
         <v/>
       </c>
       <c r="J37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$37:$AA$37))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$37:$AA$37=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$37:$AA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$37:$Y$37))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$37:$Y$37=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$37:$Y$37)))</f>
         <v/>
       </c>
       <c r="K37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$37:$AA$37))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$37:$AA$37=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$37:$AA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$37:$Y$37))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$37:$Y$37=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$37:$Y$37)))</f>
         <v/>
       </c>
       <c r="L37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$37:$AA$37))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$37:$AA$37=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$37:$AA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$37:$Y$37))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$37:$Y$37=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$37:$Y$37)))</f>
         <v/>
       </c>
     </row>
@@ -6960,23 +6686,23 @@
       <c r="E38" s="5" t="n"/>
       <c r="F38" s="5" t="n"/>
       <c r="H38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$38:$AA$38))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$38:$AA$38=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$38:$AA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$38:$Y$38))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$38:$Y$38=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$38:$Y$38)))</f>
         <v/>
       </c>
       <c r="I38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$38:$AA$38))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$38:$AA$38=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$38:$AA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$38:$Y$38))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$38:$Y$38=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$38:$Y$38)))</f>
         <v/>
       </c>
       <c r="J38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$38:$AA$38))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$38:$AA$38=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$38:$AA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$38:$Y$38))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$38:$Y$38=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$38:$Y$38)))</f>
         <v/>
       </c>
       <c r="K38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$38:$AA$38))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$38:$AA$38=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$38:$AA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$38:$Y$38))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$38:$Y$38=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$38:$Y$38)))</f>
         <v/>
       </c>
       <c r="L38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$38:$AA$38))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$38:$AA$38=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$38:$AA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$38:$Y$38))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$38:$Y$38=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$38:$Y$38)))</f>
         <v/>
       </c>
     </row>
@@ -6990,23 +6716,23 @@
       <c r="E39" s="5" t="n"/>
       <c r="F39" s="5" t="n"/>
       <c r="H39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$39:$AA$39))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$39:$AA$39=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$39:$AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$39:$Y$39))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$39:$Y$39=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$39:$Y$39)))</f>
         <v/>
       </c>
       <c r="I39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$39:$AA$39))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$39:$AA$39=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$39:$AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$39:$Y$39))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$39:$Y$39=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$39:$Y$39)))</f>
         <v/>
       </c>
       <c r="J39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$39:$AA$39))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$39:$AA$39=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$39:$AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$39:$Y$39))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$39:$Y$39=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$39:$Y$39)))</f>
         <v/>
       </c>
       <c r="K39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$39:$AA$39))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$39:$AA$39=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$39:$AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$39:$Y$39))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$39:$Y$39=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$39:$Y$39)))</f>
         <v/>
       </c>
       <c r="L39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$39:$AA$39))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$39:$AA$39=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$39:$AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$39:$Y$39))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$39:$Y$39=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$39:$Y$39)))</f>
         <v/>
       </c>
     </row>
@@ -7020,23 +6746,23 @@
       <c r="E40" s="5" t="n"/>
       <c r="F40" s="5" t="n"/>
       <c r="H40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$40:$AA$40))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$40:$AA$40=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$40:$AA$40)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$40:$Y$40))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$40:$Y$40=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$40:$Y$40)))</f>
         <v/>
       </c>
       <c r="I40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$40:$AA$40))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$40:$AA$40=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$40:$AA$40)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$40:$Y$40))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$40:$Y$40=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$40:$Y$40)))</f>
         <v/>
       </c>
       <c r="J40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$40:$AA$40))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$40:$AA$40=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$40:$AA$40)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$40:$Y$40))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$40:$Y$40=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$40:$Y$40)))</f>
         <v/>
       </c>
       <c r="K40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$40:$AA$40))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$40:$AA$40=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$40:$AA$40)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$40:$Y$40))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$40:$Y$40=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$40:$Y$40)))</f>
         <v/>
       </c>
       <c r="L40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$40:$AA$40))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$40:$AA$40=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$40:$AA$40)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$40:$Y$40))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$40:$Y$40=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$40:$Y$40)))</f>
         <v/>
       </c>
     </row>
@@ -7050,23 +6776,23 @@
       <c r="E41" s="5" t="n"/>
       <c r="F41" s="5" t="n"/>
       <c r="H41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$41:$AA$41))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$41:$AA$41=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$41:$AA$41)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$41:$Y$41))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$41:$Y$41=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$41:$Y$41)))</f>
         <v/>
       </c>
       <c r="I41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$41:$AA$41))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$41:$AA$41=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$41:$AA$41)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$41:$Y$41))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$41:$Y$41=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$41:$Y$41)))</f>
         <v/>
       </c>
       <c r="J41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$41:$AA$41))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$41:$AA$41=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$41:$AA$41)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$41:$Y$41))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$41:$Y$41=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$41:$Y$41)))</f>
         <v/>
       </c>
       <c r="K41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$41:$AA$41))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$41:$AA$41=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$41:$AA$41)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$41:$Y$41))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$41:$Y$41=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$41:$Y$41)))</f>
         <v/>
       </c>
       <c r="L41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$41:$AA$41))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$41:$AA$41=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$41:$AA$41)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$41:$Y$41))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$41:$Y$41=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$41:$Y$41)))</f>
         <v/>
       </c>
     </row>
@@ -7080,23 +6806,23 @@
       <c r="E42" s="5" t="n"/>
       <c r="F42" s="5" t="n"/>
       <c r="H42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$42:$AA$42))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$42:$AA$42=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$42:$AA$42)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$42:$Y$42))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$42:$Y$42=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$42:$Y$42)))</f>
         <v/>
       </c>
       <c r="I42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$42:$AA$42))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$42:$AA$42=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$42:$AA$42)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$42:$Y$42))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$42:$Y$42=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$42:$Y$42)))</f>
         <v/>
       </c>
       <c r="J42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$42:$AA$42))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$42:$AA$42=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$42:$AA$42)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$42:$Y$42))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$42:$Y$42=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$42:$Y$42)))</f>
         <v/>
       </c>
       <c r="K42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$42:$AA$42))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$42:$AA$42=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$42:$AA$42)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$42:$Y$42))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$42:$Y$42=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$42:$Y$42)))</f>
         <v/>
       </c>
       <c r="L42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$42:$AA$42))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$42:$AA$42=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$42:$AA$42)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$42:$Y$42))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$42:$Y$42=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$42:$Y$42)))</f>
         <v/>
       </c>
     </row>
@@ -7110,23 +6836,23 @@
       <c r="E43" s="5" t="n"/>
       <c r="F43" s="5" t="n"/>
       <c r="H43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$43:$AA$43))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*(Marks!$B$43:$AA$43=1))/SUMPRODUCT((Marks!$B$2:$AA$2=H$3)*ISNUMBER(Marks!$B$43:$AA$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$43:$Y$43))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*(Marks!$B$43:$Y$43=1))/SUMPRODUCT((Marks!$B$2:$Y$2=H$3)*ISNUMBER(Marks!$B$43:$Y$43)))</f>
         <v/>
       </c>
       <c r="I43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$43:$AA$43))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*(Marks!$B$43:$AA$43=1))/SUMPRODUCT((Marks!$B$2:$AA$2=I$3)*ISNUMBER(Marks!$B$43:$AA$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$43:$Y$43))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*(Marks!$B$43:$Y$43=1))/SUMPRODUCT((Marks!$B$2:$Y$2=I$3)*ISNUMBER(Marks!$B$43:$Y$43)))</f>
         <v/>
       </c>
       <c r="J43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$43:$AA$43))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*(Marks!$B$43:$AA$43=1))/SUMPRODUCT((Marks!$B$2:$AA$2=J$3)*ISNUMBER(Marks!$B$43:$AA$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$43:$Y$43))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*(Marks!$B$43:$Y$43=1))/SUMPRODUCT((Marks!$B$2:$Y$2=J$3)*ISNUMBER(Marks!$B$43:$Y$43)))</f>
         <v/>
       </c>
       <c r="K43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$43:$AA$43))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*(Marks!$B$43:$AA$43=1))/SUMPRODUCT((Marks!$B$2:$AA$2=K$3)*ISNUMBER(Marks!$B$43:$AA$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$43:$Y$43))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*(Marks!$B$43:$Y$43=1))/SUMPRODUCT((Marks!$B$2:$Y$2=K$3)*ISNUMBER(Marks!$B$43:$Y$43)))</f>
         <v/>
       </c>
       <c r="L43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$43:$AA$43))=0,"",SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*(Marks!$B$43:$AA$43=1))/SUMPRODUCT((Marks!$B$2:$AA$2=L$3)*ISNUMBER(Marks!$B$43:$AA$43)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$43:$Y$43))=0,"",SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*(Marks!$B$43:$Y$43=1))/SUMPRODUCT((Marks!$B$2:$Y$2=L$3)*ISNUMBER(Marks!$B$43:$Y$43)))</f>
         <v/>
       </c>
     </row>

</xml_diff>